<commit_message>
Refresh relevance focus and Radar evidence
</commit_message>
<xml_diff>
--- a/Relevance Stuff/relevance_stuff.xlsx
+++ b/Relevance Stuff/relevance_stuff.xlsx
@@ -21977,71 +21977,71 @@
     </row>
     <row r="24">
       <c r="A24" s="3">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">AI Governance and Geopolitics</t>
+          <t xml:space="preserve">EU-Africa cooperation in research and innovation</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-05-27</t>
+          <t xml:space="preserve">2026-10-27T12:00Z</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">CERRE — Centre on Regulation in Europe</t>
+          <t xml:space="preserve">EU Research &amp; Innovation</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main A</t>
+          <t xml:space="preserve">Main C</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">United States; China</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Americas; Asia &amp; Pacific</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transnational R&amp;I and innovation policy; EU-facing technology standards / regulatory alignment</t>
+          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement; Equitable international research partnerships</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business / industry</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: United States, China; issue: Transnational R&amp;I and innovation policy, EU-facing technology standards / regulatory alignment</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: EU external R&amp;I partnerships / enlargement, Equitable international research partnerships</t>
         </is>
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Report finds jurisdictions share AI policy objectives but differ in state control and tolerance of private power.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="M24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">This may change Europe's relative research and innovation capacity in technologies that increasingly shape geopolitical power.</t>
         </is>
       </c>
       <c r="N24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">keep</t>
+          <t xml:space="preserve">provisional</t>
         </is>
       </c>
       <c r="O24" s="3" t="inlineStr">
@@ -22061,12 +22061,12 @@
       </c>
       <c r="R24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">CERRE — Centre on Regulation in Europe</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="S24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://cerre.eu/wp-content/uploads/2026/05/CERRE_AI-Governance-and-Geopolitics-1.pdf</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMiqAJBVV95cUxQaWNKNUFoZWJjS0o5dWVrVzJ2ZzhKSWxkSlNxekhJV196N3RzTjNITjNlbFNFbFJtZVg2ekxteVRjN0oyMEpaUlJXRk5URUVzc3czX0RDTDg3QXRPdzJ5VUZtSTlIbmF1Z0JnZXlKNlg0RTZ4aGFfVnVTLWRwQmJOMjlycjRWclBfdGphc2ZNRlNydTRzWENKVnVyRFlJUURGOXBjcHJGdWZXX1BFTlBnOEFfVUJYQzUyQ0FsczYwSDNjOEhwTVBVRjdOSUFjX1N0QUFKb1JDazdfQWs3LVd1d0NrYXNDTktXWVM0NUxHcm9ld1BZeUZHdXFBSkdFcjRXMnhVYk9nSnd4Z2ZCRkNfVy1tcXFoaW9wU05QeDlIWTJBN0hsSVBsdA?oc=5</t>
         </is>
       </c>
     </row>
@@ -22076,17 +22076,17 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are we ready to handle PV waste? A review of PV recycling regulations in Europe, the United States, China, and India</t>
+          <t xml:space="preserve">AI Governance and Geopolitics</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-05</t>
+          <t xml:space="preserve">2026-05-27</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Energy Sustainability and Society</t>
+          <t xml:space="preserve">CERRE — Centre on Regulation in Europe</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -22101,7 +22101,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">United States; China; India</t>
+          <t xml:space="preserve">United States; China</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -22111,22 +22111,22 @@
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Transnational R&amp;I and innovation policy; EU-facing technology standards / regulatory alignment</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Business / industry</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: United States, China, India; issue: EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: United States, China; issue: Transnational R&amp;I and innovation policy, EU-facing technology standards / regulatory alignment</t>
         </is>
       </c>
       <c r="L25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The four jurisdictions differ sharply in regulatory readiness for the coming wave of photovoltaic waste.</t>
+          <t xml:space="preserve">Report finds jurisdictions share AI policy objectives but differ in state control and tolerance of private power.</t>
         </is>
       </c>
       <c r="M25" s="3" t="inlineStr">
@@ -22136,7 +22136,7 @@
       </c>
       <c r="N25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">review</t>
+          <t xml:space="preserve">keep</t>
         </is>
       </c>
       <c r="O25" s="3" t="inlineStr">
@@ -22146,22 +22146,22 @@
       </c>
       <c r="P25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14T07:26:39Z</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">worker-b-20260914T062900Z-b105dc9c7d1b</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="R25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Umer Shahzad, Cristina Irene Mihai, Ian Marius Peters</t>
+          <t xml:space="preserve">CERRE — Centre on Regulation in Europe</t>
         </is>
       </c>
       <c r="S25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://doi.org/10.1186/s13705-026-00595-7</t>
+          <t xml:space="preserve">https://cerre.eu/wp-content/uploads/2026/05/CERRE_AI-Governance-and-Geopolitics-1.pdf</t>
         </is>
       </c>
     </row>
@@ -22171,17 +22171,17 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Japan's security policy under Prime Minister Takaichi</t>
+          <t xml:space="preserve">Are we ready to handle PV waste? A review of PV recycling regulations in Europe, the United States, China, and India</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-03</t>
+          <t xml:space="preserve">2026-08-05</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Finnish Institute of International Affairs</t>
+          <t xml:space="preserve">Energy Sustainability and Society</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -22196,7 +22196,7 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">United States; Indonesia; Australia; China</t>
+          <t xml:space="preserve">United States; China; India</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
@@ -22206,7 +22206,7 @@
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research security / dual use; Australia strategic reorientation to Europe</t>
+          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
@@ -22216,17 +22216,17 @@
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: United States, Indonesia, Australia, China; issue: Research security / dual use, Australia strategic reorientation to Europe</t>
+          <t xml:space="preserve">Region: United States, China, India; issue: EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Takaichi is expanding defence exports and dual-use R&amp;D, turning Japan from arms importer into co-producer.</t>
+          <t xml:space="preserve">The four jurisdictions differ sharply in regulatory readiness for the coming wave of photovoltaic waste.</t>
         </is>
       </c>
       <c r="M26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Japan's move to co-production creates concrete openings for European defence-technology and industrial partnerships.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="N26" s="3" t="inlineStr">
@@ -22241,42 +22241,42 @@
       </c>
       <c r="P26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">2026-09-14T07:26:39Z</t>
         </is>
       </c>
       <c r="Q26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">worker-b-20260914T062900Z-b105dc9c7d1b</t>
         </is>
       </c>
       <c r="R26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bart Gaens</t>
+          <t xml:space="preserve">Umer Shahzad, Cristina Irene Mihai, Ian Marius Peters</t>
         </is>
       </c>
       <c r="S26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://fiia.fi/wp-content/uploads/2026/09/BP441_Japans-security-policy-under-Prime-Minister-Takaichi.pdf</t>
+          <t xml:space="preserve">https://doi.org/10.1186/s13705-026-00595-7</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ukraine within Eureka’s innovation landscape</t>
+          <t xml:space="preserve">Japan's security policy under Prime Minister Takaichi</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-03-09</t>
+          <t xml:space="preserve">2026-09-03</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EUREKA</t>
+          <t xml:space="preserve">Finnish Institute of International Affairs</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -22291,17 +22291,17 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ukraine</t>
+          <t xml:space="preserve">United States; Indonesia; Australia; China</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Europe — enlargement</t>
+          <t xml:space="preserve">Americas; Asia &amp; Pacific</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transnational R&amp;I and innovation policy; EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Research security / dual use; Australia strategic reorientation to Europe</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
@@ -22311,22 +22311,22 @@
       </c>
       <c r="K27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: Ukraine; issue: Transnational R&amp;I and innovation policy, EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: United States, Indonesia, Australia, China; issue: Research security / dual use, Australia strategic reorientation to Europe</t>
         </is>
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Describes Ukraine's membership since 2006 as a channel for internationalising its research system during war.</t>
+          <t xml:space="preserve">Takaichi is expanding defence exports and dual-use R&amp;D, turning Japan from arms importer into co-producer.</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Japan's move to co-production creates concrete openings for European defence-technology and industrial partnerships.</t>
         </is>
       </c>
       <c r="N27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">keep</t>
+          <t xml:space="preserve">review</t>
         </is>
       </c>
       <c r="O27" s="3" t="inlineStr">
@@ -22346,12 +22346,12 @@
       </c>
       <c r="R27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EUREKA</t>
+          <t xml:space="preserve">Bart Gaens</t>
         </is>
       </c>
       <c r="S27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.eurekanetwork.org/impact/ukraine-within-eurekas-innovation-landscape/</t>
+          <t xml:space="preserve">https://fiia.fi/wp-content/uploads/2026/09/BP441_Japans-security-policy-under-Prime-Minister-Takaichi.pdf</t>
         </is>
       </c>
     </row>
@@ -22361,17 +22361,17 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU and North Macedonia hold third Joint Research and Innovation Committee meeting</t>
+          <t xml:space="preserve">Ukraine within Eureka’s innovation landscape</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-04-23</t>
+          <t xml:space="preserve">2026-03-09</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ERA Portal Austria</t>
+          <t xml:space="preserve">EUREKA</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
@@ -22386,7 +22386,7 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">North Macedonia</t>
+          <t xml:space="preserve">Ukraine</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
@@ -22406,17 +22406,17 @@
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: North Macedonia; issue: Transnational R&amp;I and innovation policy, EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: Ukraine; issue: Transnational R&amp;I and innovation policy, EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The joint R&amp;I committee reviewed Horizon participation, EU initiatives and North Macedonia’s R&amp;I policy updates.</t>
+          <t xml:space="preserve">Describes Ukraine's membership since 2006 as a channel for internationalising its research system during war.</t>
         </is>
       </c>
       <c r="M28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Joint committees provide the governance channel through which associated-country research cooperation is maintained.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="N28" s="3" t="inlineStr">
@@ -22441,12 +22441,12 @@
       </c>
       <c r="R28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ERA Portal Austria</t>
+          <t xml:space="preserve">EUREKA</t>
         </is>
       </c>
       <c r="S28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://era.gv.at/news-items/eu-and-north-macedonia-hold-third-joint-research-and-innovation-committee-meeting/</t>
+          <t xml:space="preserve">https://www.eurekanetwork.org/impact/ukraine-within-eurekas-innovation-landscape/</t>
         </is>
       </c>
     </row>
@@ -22456,42 +22456,42 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU pursues closer Israel ties on air defense and space</t>
+          <t xml:space="preserve">EU and North Macedonia hold third Joint Research and Innovation Committee meeting</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08T15:00Z</t>
+          <t xml:space="preserve">2026-04-23</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Politico Europe</t>
+          <t xml:space="preserve">ERA Portal Austria</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main C</t>
+          <t xml:space="preserve">Main A</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Israel</t>
+          <t xml:space="preserve">North Macedonia</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Middle East</t>
+          <t xml:space="preserve">Europe — enlargement</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research security / dual use; Transnational R&amp;I and innovation policy</t>
+          <t xml:space="preserve">Transnational R&amp;I and innovation policy; EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
@@ -22501,17 +22501,17 @@
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: Israel; issue: Research security / dual use, Transnational R&amp;I and innovation policy</t>
+          <t xml:space="preserve">Region: North Macedonia; issue: Transnational R&amp;I and innovation policy, EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Israel's space agency chief met the EU research and innovation commissioner for talks on AI and robotics.</t>
+          <t xml:space="preserve">The joint R&amp;I committee reviewed Horizon participation, EU initiatives and North Macedonia’s R&amp;I policy updates.</t>
         </is>
       </c>
       <c r="M29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dual-use technology cooperation is being rebuilt after years of effective EU-Israel disengagement.</t>
+          <t xml:space="preserve">Joint committees provide the governance channel through which associated-country research cooperation is maintained.</t>
         </is>
       </c>
       <c r="N29" s="3" t="inlineStr">
@@ -22536,57 +22536,57 @@
       </c>
       <c r="R29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ERA Portal Austria</t>
         </is>
       </c>
       <c r="S29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMifEFVX3lxTFBMdlpkQThhcEIxMHVXa2xWQk1Ed0NyLTNicFhzOGFFd0doTjFQZm9md3NuTzlkY0pUQzUtU0FLTm5pRy0wMVZJcUxNNjEzSm5UdGlHNG5XdlNVZXB4cElUQUlka1FpbV9rNXEtREoydWxVV3pWbGdsUUlvd1Q?oc=5</t>
+          <t xml:space="preserve">https://era.gv.at/news-items/eu-and-north-macedonia-hold-third-joint-research-and-innovation-committee-meeting/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transatlantic cooperation on AI and national security</t>
+          <t xml:space="preserve">EU pursues closer Israel ties on air defense and space</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-04-09</t>
+          <t xml:space="preserve">2026-09-08T15:00Z</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">CERRE — Centre on Regulation in Europe</t>
+          <t xml:space="preserve">Politico Europe</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main A</t>
+          <t xml:space="preserve">Main C</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">China</t>
+          <t xml:space="preserve">Israel</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asia &amp; Pacific</t>
+          <t xml:space="preserve">Middle East</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research security / dual use</t>
+          <t xml:space="preserve">Research security / dual use; Transnational R&amp;I and innovation policy</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr">
@@ -22596,17 +22596,17 @@
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: China; issue: Research security / dual use</t>
+          <t xml:space="preserve">Region: Israel; issue: Research security / dual use, Transnational R&amp;I and innovation policy</t>
         </is>
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Issue paper identifies US policy uncertainty, European China positions and asymmetric leverage as barriers to deeper AI-security cooperation.</t>
+          <t xml:space="preserve">Israel's space agency chief met the EU research and innovation commissioner for talks on AI and robotics.</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Export controls can constrain European AI competitiveness while creating pressure for pragmatic transatlantic coordination.</t>
+          <t xml:space="preserve">Dual-use technology cooperation is being rebuilt after years of effective EU-Israel disengagement.</t>
         </is>
       </c>
       <c r="N30" s="3" t="inlineStr">
@@ -22631,12 +22631,12 @@
       </c>
       <c r="R30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Antonio Calcara, Zach Meyers</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="S30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://cerre.eu/wp-content/uploads/2026/04/CERRE_Transatlantic-cooperation-on-AI-and-national-security.pdf</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMifEFVX3lxTFBMdlpkQThhcEIxMHVXa2xWQk1Ed0NyLTNicFhzOGFFd0doTjFQZm9md3NuTzlkY0pUQzUtU0FLTm5pRy0wMVZJcUxNNjEzSm5UdGlHNG5XdlNVZXB4cElUQUlka1FpbV9rNXEtREoydWxVV3pWbGdsUUlvd1Q?oc=5</t>
         </is>
       </c>
     </row>
@@ -22646,17 +22646,17 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Universities as the Next Counterintelligence Battleground in Geopolitical Contests</t>
+          <t xml:space="preserve">Transatlantic cooperation on AI and national security</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-04-15</t>
+          <t xml:space="preserve">2026-04-09</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Global Policy</t>
+          <t xml:space="preserve">CERRE — Centre on Regulation in Europe</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -22671,12 +22671,12 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">United States; Canada</t>
+          <t xml:space="preserve">China</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Americas</t>
+          <t xml:space="preserve">Asia &amp; Pacific</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -22686,27 +22686,27 @@
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Universities / research institutions</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: United States, Canada; issue: Research security / dual use</t>
+          <t xml:space="preserve">Region: China; issue: Research security / dual use</t>
         </is>
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The article argues universities face espionage, interference and IP theft and should adapt counterintelligence concepts to research security.</t>
+          <t xml:space="preserve">Issue paper identifies US policy uncertainty, European China positions and asymmetric leverage as barriers to deeper AI-security cooperation.</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">European governments already use research-security frameworks, but the article’s main frame is global.</t>
+          <t xml:space="preserve">Export controls can constrain European AI competitiveness while creating pressure for pragmatic transatlantic coordination.</t>
         </is>
       </c>
       <c r="N31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">review</t>
+          <t xml:space="preserve">keep</t>
         </is>
       </c>
       <c r="O31" s="3" t="inlineStr">
@@ -22716,22 +22716,22 @@
       </c>
       <c r="P31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-13T23:35:57Z</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="Q31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">worker-a-20260913T224815Z-8fd374ecdc27</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="R31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brendan Walker-Munro, Sascha‐Dominik Bachmann</t>
+          <t xml:space="preserve">Antonio Calcara, Zach Meyers</t>
         </is>
       </c>
       <c r="S31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://doi.org/10.1111/1758-5899.70167</t>
+          <t xml:space="preserve">https://cerre.eu/wp-content/uploads/2026/04/CERRE_Transatlantic-cooperation-on-AI-and-national-security.pdf</t>
         </is>
       </c>
     </row>
@@ -22741,17 +22741,17 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cleantech Innovation, Industrial Decarbonisation and Global Competition - Where the EU stand in the race towards net-zero compar</t>
+          <t xml:space="preserve">Universities as the Next Counterintelligence Battleground in Geopolitical Contests</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-23</t>
+          <t xml:space="preserve">2026-04-15</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">European Parliament</t>
+          <t xml:space="preserve">Global Policy</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -22766,42 +22766,42 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">China</t>
+          <t xml:space="preserve">United States; Canada</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asia &amp; Pacific</t>
+          <t xml:space="preserve">Americas</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Research security / dual use</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Universities / research institutions</t>
         </is>
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: China; issue: EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: United States, Canada; issue: Research security / dual use</t>
         </is>
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A European Parliament study compares EU, US and Chinese cleantech innovation, manufacturing and deployment.</t>
+          <t xml:space="preserve">The article argues universities face espionage, interference and IP theft and should adapt counterintelligence concepts to research security.</t>
         </is>
       </c>
       <c r="M32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">It identifies where European innovation strengths do and do not translate into industrial scale.</t>
+          <t xml:space="preserve">European governments already use research-security frameworks, but the article’s main frame is global.</t>
         </is>
       </c>
       <c r="N32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">keep</t>
+          <t xml:space="preserve">review</t>
         </is>
       </c>
       <c r="O32" s="3" t="inlineStr">
@@ -22811,42 +22811,42 @@
       </c>
       <c r="P32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">2026-09-13T23:35:57Z</t>
         </is>
       </c>
       <c r="Q32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">worker-a-20260913T224815Z-8fd374ecdc27</t>
         </is>
       </c>
       <c r="R32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Brendan Walker-Munro, Sascha‐Dominik Bachmann</t>
         </is>
       </c>
       <c r="S32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMilAFBVV95cUxOTWkwRkprZGk0MVlUUUxEb1FxWHphLTctdVZEZjYycFkyYmdJNDlXazFuRlM5bHhnUjdkNXpuWTNHb1pSN19obExEaFRBRjhoZXpJbHRfbnpnbDE1cTZaSnhQZFJoRm9FSE1aVXg5SU84OUlCWHdGU1pzY09BRjJaTks2NW5Ha2Z4S0w5STc5dmFmTmkw?oc=5</t>
+          <t xml:space="preserve">https://doi.org/10.1111/1758-5899.70167</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research security as a collective responsibility: empowering universities, enabling Europe</t>
+          <t xml:space="preserve">Cleantech Innovation, Industrial Decarbonisation and Global Competition - Where the EU stand in the race towards net-zero compar</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-10-27</t>
+          <t xml:space="preserve">2026-08-23</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">CESAER</t>
+          <t xml:space="preserve">European Parliament</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
@@ -22861,37 +22861,37 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">China</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Asia &amp; Pacific</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research security / dual use; EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Universities / research institutions</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Research security / dual use, EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: China; issue: EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The input note combines university practices with requests for proportionate European and national research-security support.</t>
+          <t xml:space="preserve">A European Parliament study compares EU, US and Chinese cleantech innovation, manufacturing and deployment.</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">It argues safeguards work best when researchers and institutions receive capacity, guidance and consistent rules rather than blanket restrictions.</t>
+          <t xml:space="preserve">It identifies where European innovation strengths do and do not translate into industrial scale.</t>
         </is>
       </c>
       <c r="N33" s="3" t="inlineStr">
@@ -22916,12 +22916,12 @@
       </c>
       <c r="R33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">CESAER</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="S33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.cesaer.org/publications/input-note-research-security-as-a-collective-responsibility-empowering-universities-enabling-europe/</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMilAFBVV95cUxOTWkwRkprZGk0MVlUUUxEb1FxWHphLTctdVZEZjYycFkyYmdJNDlXazFuRlM5bHhnUjdkNXpuWTNHb1pSN19obExEaFRBRjhoZXpJbHRfbnpnbDE1cTZaSnhQZFJoRm9FSE1aVXg5SU84OUlCWHdGU1pzY09BRjJaTks2NW5Ha2Z4S0w5STc5dmFmTmkw?oc=5</t>
         </is>
       </c>
     </row>
@@ -22931,27 +22931,27 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Initiative 3.2. Strengthen Research Security</t>
+          <t xml:space="preserve">Research security as a collective responsibility: empowering universities, enabling Europe</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-03-16</t>
+          <t xml:space="preserve">2025-10-27</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ERA Portal Austria</t>
+          <t xml:space="preserve">CESAER</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main C</t>
+          <t xml:space="preserve">Main A</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -22966,27 +22966,27 @@
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research security / dual use; Transnational R&amp;I and innovation policy</t>
+          <t xml:space="preserve">Research security / dual use; EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Universities / research institutions; Business / industry</t>
+          <t xml:space="preserve">Universities / research institutions</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Research security / dual use, Transnational R&amp;I and innovation policy</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Research security / dual use, EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Austria’s 2026–2028 ERA plan creates coordination, awareness and risk-management actions for international scientific cooperation.</t>
+          <t xml:space="preserve">The input note combines university practices with requests for proportionate European and national research-security support.</t>
         </is>
       </c>
       <c r="M34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The initiative connects EU recommendations with practical risk assessment and capacity building in Austrian research organisations.</t>
+          <t xml:space="preserve">It argues safeguards work best when researchers and institutions receive capacity, guidance and consistent rules rather than blanket restrictions.</t>
         </is>
       </c>
       <c r="N34" s="3" t="inlineStr">
@@ -23011,12 +23011,12 @@
       </c>
       <c r="R34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ERA Portal Austria</t>
+          <t xml:space="preserve">CESAER</t>
         </is>
       </c>
       <c r="S34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://era.gv.at/era/era-in-austria/national-era-action-plan-2026-2028/field-of-action-3/initiative-32-strengthen-research-security/</t>
+          <t xml:space="preserve">https://www.cesaer.org/publications/input-note-research-security-as-a-collective-responsibility-empowering-universities-enabling-europe/</t>
         </is>
       </c>
     </row>
@@ -23026,62 +23026,62 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Artificial Intelligence and Foreign Information Manipulation: Chinese and Russian approaches</t>
+          <t xml:space="preserve">Initiative 3.2. Strengthen Research Security</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-03-31</t>
+          <t xml:space="preserve">2026-03-16</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hybrid CoE — European Centre of Excellence for Countering Hybrid Threats</t>
+          <t xml:space="preserve">ERA Portal Austria</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main A</t>
+          <t xml:space="preserve">Main C</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">China</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asia &amp; Pacific</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Research security / dual use; Transnational R&amp;I and innovation policy</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Universities / research institutions; Business / industry</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: China; issue: EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Research security / dual use, Transnational R&amp;I and innovation policy</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The paper compares how China and Russia use AI for influence operations, data gathering, targeting and content production.</t>
+          <t xml:space="preserve">Austria’s 2026–2028 ERA plan creates coordination, awareness and risk-management actions for international scientific cooperation.</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">AI can scale hostile information operations against European and allied democratic decision-making.</t>
+          <t xml:space="preserve">The initiative connects EU recommendations with practical risk assessment and capacity building in Austrian research organisations.</t>
         </is>
       </c>
       <c r="N35" s="3" t="inlineStr">
@@ -23106,12 +23106,12 @@
       </c>
       <c r="R35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Heidi Hanhijärvi</t>
+          <t xml:space="preserve">ERA Portal Austria</t>
         </is>
       </c>
       <c r="S35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.hybridcoe.fi/wp-content/uploads/2026/03/Artificial-Intelligence-and-Foreign-Information-Manipulation-Hybrid-CoE-Paper-29.pdf</t>
+          <t xml:space="preserve">https://era.gv.at/era/era-in-austria/national-era-action-plan-2026-2028/field-of-action-3/initiative-32-strengthen-research-security/</t>
         </is>
       </c>
     </row>
@@ -23121,37 +23121,37 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALLEA Contributes to High-Level Discussions on the Role of Science in Ukraine’s Recovery</t>
+          <t xml:space="preserve">Artificial Intelligence and Foreign Information Manipulation: Chinese and Russian approaches</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-27</t>
+          <t xml:space="preserve">2026-03-31</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALLEA</t>
+          <t xml:space="preserve">Hybrid CoE — European Centre of Excellence for Countering Hybrid Threats</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main C</t>
+          <t xml:space="preserve">Main A</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ukraine</t>
+          <t xml:space="preserve">China</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Europe — enlargement</t>
+          <t xml:space="preserve">Asia &amp; Pacific</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
@@ -23166,17 +23166,17 @@
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: Ukraine; issue: EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: China; issue: EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">European academies joined the first High-Level Steering Committee and signed the Gdansk Declaration on Ukrainian science.</t>
+          <t xml:space="preserve">The paper compares how China and Russia use AI for influence operations, data gathering, targeting and content production.</t>
         </is>
       </c>
       <c r="M36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sets a coordinated international framework for rebuilding Ukraine's research system.</t>
+          <t xml:space="preserve">AI can scale hostile information operations against European and allied democratic decision-making.</t>
         </is>
       </c>
       <c r="N36" s="3" t="inlineStr">
@@ -23201,12 +23201,12 @@
       </c>
       <c r="R36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALLEA</t>
+          <t xml:space="preserve">Heidi Hanhijärvi</t>
         </is>
       </c>
       <c r="S36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://allea.org/allea-contributes-to-high-level-discussions-on-the-role-of-science-in-ukraines-recovery/</t>
+          <t xml:space="preserve">https://www.hybridcoe.fi/wp-content/uploads/2026/03/Artificial-Intelligence-and-Foreign-Information-Manipulation-Hybrid-CoE-Paper-29.pdf</t>
         </is>
       </c>
     </row>
@@ -23216,62 +23216,62 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU and US critical raw materials strategies: EU-US Explainer</t>
+          <t xml:space="preserve">ALLEA Contributes to High-Level Discussions on the Role of Science in Ukraine’s Recovery</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-07-16T07:00Z</t>
+          <t xml:space="preserve">2026-06-27</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">European Parliament</t>
+          <t xml:space="preserve">ALLEA</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main A</t>
+          <t xml:space="preserve">Main C</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Ukraine</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Europe — enlargement</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Critical raw materials × R&amp;I / technology; EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business / industry</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology, EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: Ukraine; issue: EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A European Parliament briefing compares EU and US critical-raw-material strategies, dependencies and policy tools.</t>
+          <t xml:space="preserve">European academies joined the first High-Level Steering Committee and signed the Gdansk Declaration on Ukrainian science.</t>
         </is>
       </c>
       <c r="M37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">It documents structural supply risks that shape European research, industry and strategic autonomy.</t>
+          <t xml:space="preserve">Sets a coordinated international framework for rebuilding Ukraine's research system.</t>
         </is>
       </c>
       <c r="N37" s="3" t="inlineStr">
@@ -23296,12 +23296,12 @@
       </c>
       <c r="R37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ALLEA</t>
         </is>
       </c>
       <c r="S37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMifkFVX3lxTFA3d1VZbmNrSnJ1MW5xdnNzdjBBRzMzeTF4VUhMeXdzb3VXeG9yZ2Z1aDdTZEFRZ05JNjFXN0JRMW93a0dtWlI2OG1Jd1hyVTNqaWFEWU9veDZUQzQxLWdIcjUwR1RHRFNZenRyWkUxR1hHaWZieE03MUNzU3FUZw?oc=5</t>
+          <t xml:space="preserve">https://allea.org/allea-contributes-to-high-level-discussions-on-the-role-of-science-in-ukraines-recovery/</t>
         </is>
       </c>
     </row>
@@ -23311,7 +23311,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">India starts formal talks on Horizon Europe association</t>
+          <t xml:space="preserve">EU and US critical raw materials strategies: EU-US Explainer</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -23321,52 +23321,52 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Science|Business</t>
+          <t xml:space="preserve">European Parliament</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main C</t>
+          <t xml:space="preserve">Main A</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">India</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asia &amp; Pacific</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Critical raw materials × R&amp;I / technology; EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Business / industry</t>
         </is>
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: India; issue: EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology, EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The EU and India began formal negotiations on Horizon Europe association after their July Trade and Technology Council meeting.</t>
+          <t xml:space="preserve">A European Parliament briefing compares EU and US critical-raw-material strategies, dependencies and policy tools.</t>
         </is>
       </c>
       <c r="M38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Association would make Indian researchers directly eligible for EU programme funding in return for a national contribution.</t>
+          <t xml:space="preserve">It documents structural supply risks that shape European research, industry and strategic autonomy.</t>
         </is>
       </c>
       <c r="N38" s="3" t="inlineStr">
@@ -23396,7 +23396,7 @@
       </c>
       <c r="S38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMiogFBVV95cUxPcmRseE5uVWZkcEplU01GOUlLVjd5djhjQ0xJbTRHTmZTNUh5R0xsRWdGOTF5amsya2JaVDFUZHJWVHV2QlVKNEQ1S3NGT2xlZVJqclZBZGlLS25BaHBDRWVMSlNLMmItMnJPRVVJU1RCSHZCZ2FPVnk2SDUxR29XMExzTWpKajJyN1h1VndlbTFibENUOHpHaGFuMy0taUdMcFE?oc=5</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMifkFVX3lxTFA3d1VZbmNrSnJ1MW5xdnNzdjBBRzMzeTF4VUhMeXdzb3VXeG9yZ2Z1aDdTZEFRZ05JNjFXN0JRMW93a0dtWlI2OG1Jd1hyVTNqaWFEWU9veDZUQzQxLWdIcjUwR1RHRFNZenRyWkUxR1hHaWZieE03MUNzU3FUZw?oc=5</t>
         </is>
       </c>
     </row>
@@ -23406,12 +23406,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data Corner: Indian participation in Horizon Europe</t>
+          <t xml:space="preserve">India starts formal talks on Horizon Europe association</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-01</t>
+          <t xml:space="preserve">2026-07-16T07:00Z</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -23456,12 +23456,12 @@
       </c>
       <c r="L39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Indian organisations already participate in Horizon Europe, with €3.4 million in EU funding reported before formal association.</t>
+          <t xml:space="preserve">The EU and India began formal negotiations on Horizon Europe association after their July Trade and Technology Council meeting.</t>
         </is>
       </c>
       <c r="M39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The data establish a baseline for how association could change India’s access to EU research funding.</t>
+          <t xml:space="preserve">Association would make Indian researchers directly eligible for EU programme funding in return for a national contribution.</t>
         </is>
       </c>
       <c r="N39" s="3" t="inlineStr">
@@ -23491,7 +23491,7 @@
       </c>
       <c r="S39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMiqwFBVV95cUxQRVhFMmIxN3AtRkFXelpLaDBYejd0emlMam9sc2FBZWhoTHpHdV90TjNpYTFHc3d4WXo5UmhzUHpKMUpBTFNZMkU0SlRiZWpjSktfZlROVWN2SkI5QXhkbjZCN0ZlYXB6UkptOXoxOElncHZrVmxodEo0SGlSUnVzZmNkcTd5WXpLLVVKSFlVMWpJaWFzVTVxTHhDZzQwRHFOLVJiYUxoTXRkS28?oc=5</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMiogFBVV95cUxPcmRseE5uVWZkcEplU01GOUlLVjd5djhjQ0xJbTRHTmZTNUh5R0xsRWdGOTF5amsya2JaVDFUZHJWVHV2QlVKNEQ1S3NGT2xlZVJqclZBZGlLS25BaHBDRWVMSlNLMmItMnJPRVVJU1RCSHZCZ2FPVnk2SDUxR29XMExzTWpKajJyN1h1VndlbTFibENUOHpHaGFuMy0taUdMcFE?oc=5</t>
         </is>
       </c>
     </row>
@@ -23501,17 +23501,17 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Belgian-Chinese researcher arrested over suspected theft of chip secrets</t>
+          <t xml:space="preserve">Data Corner: Indian participation in Horizon Europe</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07T15:55Z</t>
+          <t xml:space="preserve">2026-09-01</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Financial Times</t>
+          <t xml:space="preserve">Science|Business</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -23526,7 +23526,7 @@
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">China</t>
+          <t xml:space="preserve">India</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
@@ -23546,17 +23546,17 @@
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: China; issue: EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: India; issue: EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Belgian authorities arrested a semiconductor researcher suspected of misappropriating gallium-nitride technology and trade secrets.</t>
+          <t xml:space="preserve">Indian organisations already participate in Horizon Europe, with €3.4 million in EU funding reported before formal association.</t>
         </is>
       </c>
       <c r="M40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The case highlights research-security and intellectual-property risks around European advanced-semiconductor capability.</t>
+          <t xml:space="preserve">The data establish a baseline for how association could change India’s access to EU research funding.</t>
         </is>
       </c>
       <c r="N40" s="3" t="inlineStr">
@@ -23586,7 +23586,7 @@
       </c>
       <c r="S40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMihAFBVV95cUxOZkZIaURhUUM5bW9SczlEWWJtcmx4WUpIbjZnV3VpTHNtUWFhVUw1YndLNzc1Uzl2YmFvcG1zdVlkYUZDalJYdi01dm90WUJlcmUta1BCWHMtcF8xdWNUYUtFcnByRmp1dzVSOWptMHlLNU1zVVdNbjhYOWVpdUJuZXFJeno?oc=5</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMiqwFBVV95cUxQRVhFMmIxN3AtRkFXelpLaDBYejd0emlMam9sc2FBZWhoTHpHdV90TjNpYTFHc3d4WXo5UmhzUHpKMUpBTFNZMkU0SlRiZWpjSktfZlROVWN2SkI5QXhkbjZCN0ZlYXB6UkptOXoxOElncHZrVmxodEo0SGlSUnVzZmNkcTd5WXpLLVVKSFlVMWpJaWFzVTVxTHhDZzQwRHFOLVJiYUxoTXRkS28?oc=5</t>
         </is>
       </c>
     </row>
@@ -23596,17 +23596,17 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Experts call for a new approach to Neuro-AI governance - European Commission</t>
+          <t xml:space="preserve">Belgian-Chinese researcher arrested over suspected theft of chip secrets</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08T07:00Z</t>
+          <t xml:space="preserve">2026-09-07T15:55Z</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU Research &amp; Innovation</t>
+          <t xml:space="preserve">Financial Times</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
@@ -23621,17 +23621,17 @@
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">China</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Asia &amp; Pacific</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement; EU-facing technology standards / regulatory alignment</t>
+          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
@@ -23641,17 +23641,17 @@
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: EU external R&amp;I partnerships / enlargement, EU-facing technology standards / regulatory alignment</t>
+          <t xml:space="preserve">Region: China; issue: EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">European Group on Ethics in Science and New Technologies issued an infrastructure-focused Neuro-AI governance statement on 8 September 2026. It</t>
+          <t xml:space="preserve">Belgian authorities arrested a semiconductor researcher suspected of misappropriating gallium-nitride technology and trade secrets.</t>
         </is>
       </c>
       <c r="M41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">The case highlights research-security and intellectual-property risks around European advanced-semiconductor capability.</t>
         </is>
       </c>
       <c r="N41" s="3" t="inlineStr">
@@ -23681,7 +23681,7 @@
       </c>
       <c r="S41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMi2gFBVV95cUxNV25TdUhhYXBTczR1NlhodXZTc0xncTduYlVreTZkQjNBcmNjcG9rLS16TWQ5VklDc3NrYzNnOEVkd2NtdWlaZDVPUEEtZzFaNDB5aVZQcUpBVXFTNzNwbW9BTnpET0FtQlFsZWNtckFKT2hHZFRzeGx5d3NnUVEwRDJaRzZLNVBJUHhCcFdiMGZWVkM2R2xLdjJQTjRnMEFDZktmVWlrTTlrSjIxdkhFa0wtcTVuWW03c1FqTDhyMGMtSG16ejFrOVlIb3RLLVRQU3M4bzAxX3djUQ?oc=5</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMihAFBVV95cUxOZkZIaURhUUM5bW9SczlEWWJtcmx4WUpIbjZnV3VpTHNtUWFhVUw1YndLNzc1Uzl2YmFvcG1zdVlkYUZDalJYdi01dm90WUJlcmUta1BCWHMtcF8xdWNUYUtFcnByRmp1dzVSOWptMHlLNU1zVVdNbjhYOWVpdUJuZXFJeno?oc=5</t>
         </is>
       </c>
     </row>
@@ -23691,17 +23691,17 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU governments to debate a 19-partnership Horizon Europe portfolio</t>
+          <t xml:space="preserve">Experts call for a new approach to Neuro-AI governance - European Commission</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-08T15:40Z</t>
+          <t xml:space="preserve">2026-09-08T07:00Z</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Science|Business</t>
+          <t xml:space="preserve">EU Research &amp; Innovation</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -23726,7 +23726,7 @@
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transnational R&amp;I and innovation policy; EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement; EU-facing technology standards / regulatory alignment</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
@@ -23736,12 +23736,12 @@
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Transnational R&amp;I and innovation policy, EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: EU external R&amp;I partnerships / enlargement, EU-facing technology standards / regulatory alignment</t>
         </is>
       </c>
       <c r="L42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A proposal for 19 research partnerships was scheduled for member-state negotiations in October 2026.</t>
+          <t xml:space="preserve">European Group on Ethics in Science and New Technologies issued an infrastructure-focused Neuro-AI governance statement on 8 September 2026. It</t>
         </is>
       </c>
       <c r="M42" s="3" t="inlineStr">
@@ -23776,7 +23776,7 @@
       </c>
       <c r="S42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMiqwFBVV95cUxNa01CaEYwNVB3V3dxelh1LXE2c3lMNFVFNm1OYmEzYXBSZjVVRFJPSnVjUFVaUEtMcjhBekF0RXlacTVTRWxOMzdLMHJvdzVRbWdaanQ3R2JNbzNxaS1heUxiNk5EenFLdy0yZnVCNlFPNWdLUUJLOWJwUXFrR1dZOFlXYXpNeDFRaW9qM1pkQlBtRHhBdEk4bkNTQ1BKbUpLVlNDbUhpQmJ5aUU?oc=5</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMi2gFBVV95cUxNV25TdUhhYXBTczR1NlhodXZTc0xncTduYlVreTZkQjNBcmNjcG9rLS16TWQ5VklDc3NrYzNnOEVkd2NtdWlaZDVPUEEtZzFaNDB5aVZQcUpBVXFTNzNwbW9BTnpET0FtQlFsZWNtckFKT2hHZFRzeGx5d3NnUVEwRDJaRzZLNVBJUHhCcFdiMGZWVkM2R2xLdjJQTjRnMEFDZktmVWlrTTlrSjIxdkhFa0wtcTVuWW03c1FqTDhyMGMtSG16ejFrOVlIb3RLLVRQU3M4bzAxX3djUQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -23786,27 +23786,27 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Integrating circular economy and policy synergies for cost-efficient lithium-ion battery supply chains</t>
+          <t xml:space="preserve">EU governments to debate a 19-partnership Horizon Europe portfolio</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-16</t>
+          <t xml:space="preserve">2026-10-08T15:40Z</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Clean Technologies and Environmental Policy</t>
+          <t xml:space="preserve">Science|Business</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main A</t>
+          <t xml:space="preserve">Main C</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -23821,7 +23821,7 @@
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Critical raw materials × R&amp;I / technology; Transnational R&amp;I and innovation policy</t>
+          <t xml:space="preserve">Transnational R&amp;I and innovation policy; EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
@@ -23831,22 +23831,22 @@
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology, Transnational R&amp;I and innovation policy</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Transnational R&amp;I and innovation policy, EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A nine-country EU battery study finds recycling, research investment, subsidies and logistics jointly associate with supply-chain cost performance.</t>
+          <t xml:space="preserve">A proposal for 19 research partnerships was scheduled for member-state negotiations in October 2026.</t>
         </is>
       </c>
       <c r="M43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Results suggest strategic support can depend on complementary industrial research and circular-economy infrastructure.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="N43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">review</t>
+          <t xml:space="preserve">keep</t>
         </is>
       </c>
       <c r="O43" s="3" t="inlineStr">
@@ -23856,92 +23856,92 @@
       </c>
       <c r="P43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-21T17:46:38Z</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="Q43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">worker-b-20261021T171746Z-e44da281e3bc</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="R43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A. K. M. Mohsin, Md. Rashed, Markus Gerschberger, Sayed Farrukh Ahmed, Ladislav Bartuska, Christopher Schwarz, Md. Kamal Uddin</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="S43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://doi.org/10.1007/s10098-026-03613-6</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMiqwFBVV95cUxNa01CaEYwNVB3V3dxelh1LXE2c3lMNFVFNm1OYmEzYXBSZjVVRFJPSnVjUFVaUEtMcjhBekF0RXlacTVTRWxOMzdLMHJvdzVRbWdaanQ3R2JNbzNxaS1heUxiNk5EenFLdy0yZnVCNlFPNWdLUUJLOWJwUXFrR1dZOFlXYXpNeDFRaW9qM1pkQlBtRHhBdEk4bkNTQ1BKbUpLVlNDbUhpQmJ5aUU?oc=5</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Associated Countries urge EU to keep FP10 open and research-led</t>
+          <t xml:space="preserve">Integrating circular economy and policy synergies for cost-efficient lithium-ion battery supply chains</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-05-18</t>
+          <t xml:space="preserve">2026-10-16</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ERA Portal Austria</t>
+          <t xml:space="preserve">Clean Technologies and Environmental Policy</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main C</t>
+          <t xml:space="preserve">Main A</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Canada</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Americas</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transnational R&amp;I and innovation policy; EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Critical raw materials × R&amp;I / technology; Transnational R&amp;I and innovation policy</t>
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Universities / research institutions</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: Canada; issue: Transnational R&amp;I and innovation policy, EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology, Transnational R&amp;I and innovation policy</t>
         </is>
       </c>
       <c r="L44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">They demand a research-led Pillar II, an independent ERC and bottom-up Marie Sklodowska-Curie Actions.</t>
+          <t xml:space="preserve">A nine-country EU battery study finds recycling, research investment, subsidies and logistics jointly associate with supply-chain cost performance.</t>
         </is>
       </c>
       <c r="M44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The letter targets the Council during the FP10 design phase, when association terms are being set.</t>
+          <t xml:space="preserve">Results suggest strategic support can depend on complementary industrial research and circular-economy infrastructure.</t>
         </is>
       </c>
       <c r="N44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">keep</t>
+          <t xml:space="preserve">review</t>
         </is>
       </c>
       <c r="O44" s="3" t="inlineStr">
@@ -23951,37 +23951,37 @@
       </c>
       <c r="P44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">2026-10-21T17:46:38Z</t>
         </is>
       </c>
       <c r="Q44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">worker-b-20261021T171746Z-e44da281e3bc</t>
         </is>
       </c>
       <c r="R44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ERA Portal Austria (editorial)</t>
+          <t xml:space="preserve">A. K. M. Mohsin, Md. Rashed, Markus Gerschberger, Sayed Farrukh Ahmed, Ladislav Bartuska, Christopher Schwarz, Md. Kamal Uddin</t>
         </is>
       </c>
       <c r="S44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://era.gv.at/news-items/associated-countries-urge-eu-to-keep-fp10-open-and-research-led/</t>
+          <t xml:space="preserve">https://doi.org/10.1007/s10098-026-03613-6</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">LERU requests safeguards for dual-use research in FP10</t>
+          <t xml:space="preserve">Associated Countries urge EU to keep FP10 open and research-led</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-05-21</t>
+          <t xml:space="preserve">2026-05-18</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -23991,47 +23991,47 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main A</t>
+          <t xml:space="preserve">Main C</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Canada</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Americas</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research security / dual use; Transnational R&amp;I and innovation policy; EU-facing technology standards / regulatory alignment</t>
+          <t xml:space="preserve">Transnational R&amp;I and innovation policy; EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Universities / research institutions</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Research security / dual use, Transnational R&amp;I and innovation policy, EU-facing technology standards / regulatory alignment</t>
+          <t xml:space="preserve">Region: Canada; issue: Transnational R&amp;I and innovation policy, EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">LERU wants clear, targeted dual-use safeguards while preserving frontier research and international scientific cooperation.</t>
+          <t xml:space="preserve">They demand a research-led Pillar II, an independent ERC and bottom-up Marie Sklodowska-Curie Actions.</t>
         </is>
       </c>
       <c r="M45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overbroad security rules could discourage collaboration and basic research without targeting genuine risks.</t>
+          <t xml:space="preserve">The letter targets the Council during the FP10 design phase, when association terms are being set.</t>
         </is>
       </c>
       <c r="N45" s="3" t="inlineStr">
@@ -24056,12 +24056,12 @@
       </c>
       <c r="R45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ERA Portal Austria</t>
+          <t xml:space="preserve">ERA Portal Austria (editorial)</t>
         </is>
       </c>
       <c r="S45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://era.gv.at/news-items/leru-urges-safeguards-for-dual-use-research-in-fp10/</t>
+          <t xml:space="preserve">https://era.gv.at/news-items/associated-countries-urge-eu-to-keep-fp10-open-and-research-led/</t>
         </is>
       </c>
     </row>
@@ -24071,17 +24071,17 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">R&amp;I needs to reduce dependencies on critical raw materials through advanced materials in passenger vehicles</t>
+          <t xml:space="preserve">LERU requests safeguards for dual-use research in FP10</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-18</t>
+          <t xml:space="preserve">2026-05-21</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">European Commission, Joint Research Centre (JRC)</t>
+          <t xml:space="preserve">ERA Portal Austria</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -24106,7 +24106,7 @@
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Critical raw materials × R&amp;I / technology; Transnational R&amp;I and innovation policy; EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Research security / dual use; Transnational R&amp;I and innovation policy; EU-facing technology standards / regulatory alignment</t>
         </is>
       </c>
       <c r="J46" s="3" t="inlineStr">
@@ -24116,17 +24116,17 @@
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology, Transnational R&amp;I and innovation policy, EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Research security / dual use, Transnational R&amp;I and innovation policy, EU-facing technology standards / regulatory alignment</t>
         </is>
       </c>
       <c r="L46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mature alternatives can cut gallium, palladium, beryllium, magnesium and other critical materials in specific car parts; none is universal.</t>
+          <t xml:space="preserve">LERU wants clear, targeted dual-use safeguards while preserving frontier research and international scientific cooperation.</t>
         </is>
       </c>
       <c r="M46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mature substitutes chiefly need qualification testing and pilot-line access; the findings can inform EU research programming and materials legislation.</t>
+          <t xml:space="preserve">Overbroad security rules could discourage collaboration and basic research without targeting genuine risks.</t>
         </is>
       </c>
       <c r="N46" s="3" t="inlineStr">
@@ -24151,37 +24151,37 @@
       </c>
       <c r="R46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fernando Coelho; Awais Ikram; Filipa M. Oliveira; Stefanos Mourdikoudis; David Pennington</t>
+          <t xml:space="preserve">ERA Portal Austria</t>
         </is>
       </c>
       <c r="S46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://publications.jrc.ec.europa.eu/repository/handle/JRC148265?mode=full</t>
+          <t xml:space="preserve">https://era.gv.at/news-items/leru-urges-safeguards-for-dual-use-research-in-fp10/</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Position Paper “Past, present, and future of the European Research &amp; Innovation Framework programmes 2014-2027” | Coimbra</t>
+          <t xml:space="preserve">R&amp;I needs to reduce dependencies on critical raw materials through advanced materials in passenger vehicles</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2023-01-01</t>
+          <t xml:space="preserve">2026-09-18</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Coimbra Group</t>
+          <t xml:space="preserve">European Commission, Joint Research Centre (JRC)</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historical</t>
+          <t xml:space="preserve">Main A</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
@@ -24201,32 +24201,32 @@
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Critical raw materials × R&amp;I / technology; Transnational R&amp;I and innovation policy; EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Universities / research institutions</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology, Transnational R&amp;I and innovation policy, EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Coimbra Group reviews Horizon 2020 and Horizon Europe and recommends changes to future programme design.</t>
+          <t xml:space="preserve">Mature alternatives can cut gallium, palladium, beryllium, magnesium and other critical materials in specific car parts; none is universal.</t>
         </is>
       </c>
       <c r="M47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">University experience can reveal operational programme frictions, though the source represents stakeholder interests.</t>
+          <t xml:space="preserve">Mature substitutes chiefly need qualification testing and pilot-line access; the findings can inform EU research programming and materials legislation.</t>
         </is>
       </c>
       <c r="N47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">review</t>
+          <t xml:space="preserve">keep</t>
         </is>
       </c>
       <c r="O47" s="3" t="inlineStr">
@@ -24236,22 +24236,22 @@
       </c>
       <c r="P47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-26T05:34:15Z</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="Q47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">worker-b-20260926T041925Z-4706ad515738</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="R47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Fernando Coelho; Awais Ikram; Filipa M. Oliveira; Stefanos Mourdikoudis; David Pennington</t>
         </is>
       </c>
       <c r="S47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.coimbra-group.eu/wp-content/uploads/Coimbra-Group-Position-Paper-23Feb.pdf</t>
+          <t xml:space="preserve">https://publications.jrc.ec.europa.eu/repository/handle/JRC148265?mode=full</t>
         </is>
       </c>
     </row>
@@ -24261,17 +24261,17 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Critical raw materials, circular economy, sustainable development: EU policy reflections for future research and innovation</t>
+          <t xml:space="preserve">Position Paper “Past, present, and future of the European Research &amp; Innovation Framework programmes 2014-2027” | Coimbra</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-04-01</t>
+          <t xml:space="preserve">2023-01-01</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resources, Conservation and Recycling</t>
+          <t xml:space="preserve">Coimbra Group</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -24296,27 +24296,27 @@
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Critical raw materials × R&amp;I / technology</t>
+          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Universities / research institutions</t>
         </is>
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A JRC perspective evaluates EU circular-economy policy and critical-material recycling needs in strategic technologies.</t>
+          <t xml:space="preserve">The Coimbra Group reviews Horizon 2020 and Horizon Europe and recommends changes to future programme design.</t>
         </is>
       </c>
       <c r="M48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU innovation research priorities, material dependencies and circularity of strategic technologies are the focus of the analysis.</t>
+          <t xml:space="preserve">University experience can reveal operational programme frictions, though the source represents stakeholder interests.</t>
         </is>
       </c>
       <c r="N48" s="3" t="inlineStr">
@@ -24331,22 +24331,22 @@
       </c>
       <c r="P48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-28T13:03:44Z</t>
+          <t xml:space="preserve">2026-09-26T05:34:15Z</t>
         </is>
       </c>
       <c r="Q48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">worker-a-20261028T124131Z-6ab6d841b916</t>
+          <t xml:space="preserve">worker-b-20260926T041925Z-4706ad515738</t>
         </is>
       </c>
       <c r="R48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brian Baldassarre; Samuel Carrara</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="S48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://doi.org/10.1016/j.resconrec.2024.108060</t>
+          <t xml:space="preserve">https://www.coimbra-group.eu/wp-content/uploads/Coimbra-Group-Position-Paper-23Feb.pdf</t>
         </is>
       </c>
     </row>
@@ -24356,22 +24356,22 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Input note 'Clarifying and optimising civil, dual-use and defence research and innovation in future EU funding programmes'</t>
+          <t xml:space="preserve">Critical raw materials, circular economy, sustainable development: EU policy reflections for future research and innovation</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-03-26</t>
+          <t xml:space="preserve">2025-04-01</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">CESAER</t>
+          <t xml:space="preserve">Resources, Conservation and Recycling</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main A</t>
+          <t xml:space="preserve">Historical</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
@@ -24391,32 +24391,32 @@
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research security / dual use</t>
+          <t xml:space="preserve">Critical raw materials × R&amp;I / technology</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Universities / research institutions</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Research security / dual use</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology</t>
         </is>
       </c>
       <c r="L49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The note sets out concrete proposals for clarifying how civil, dual-use and defence R&amp;I are positioned in EU programmes.</t>
+          <t xml:space="preserve">A JRC perspective evaluates EU circular-economy policy and critical-material recycling needs in strategic technologies.</t>
         </is>
       </c>
       <c r="M49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shapes how universities can participate in EU defence-adjacent research funding.</t>
+          <t xml:space="preserve">EU innovation research priorities, material dependencies and circularity of strategic technologies are the focus of the analysis.</t>
         </is>
       </c>
       <c r="N49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">keep</t>
+          <t xml:space="preserve">review</t>
         </is>
       </c>
       <c r="O49" s="3" t="inlineStr">
@@ -24426,22 +24426,22 @@
       </c>
       <c r="P49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">2026-10-28T13:03:44Z</t>
         </is>
       </c>
       <c r="Q49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">worker-a-20261028T124131Z-6ab6d841b916</t>
         </is>
       </c>
       <c r="R49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">CESAER</t>
+          <t xml:space="preserve">Brian Baldassarre; Samuel Carrara</t>
         </is>
       </c>
       <c r="S49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.cesaer.org/publications/clarifying-and-optimising-civil-dual-use-and-defence-research-and-innovation-in-future-eu-funding-programmes/</t>
+          <t xml:space="preserve">https://doi.org/10.1016/j.resconrec.2024.108060</t>
         </is>
       </c>
     </row>
@@ -24451,17 +24451,17 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research security</t>
+          <t xml:space="preserve">Input note 'Clarifying and optimising civil, dual-use and defence research and innovation in future EU funding programmes'</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-19</t>
+          <t xml:space="preserve">2026-03-26</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research Council of Finland</t>
+          <t xml:space="preserve">CESAER</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
@@ -24491,7 +24491,7 @@
       </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Universities / research institutions</t>
         </is>
       </c>
       <c r="K50" s="3" t="inlineStr">
@@ -24501,12 +24501,12 @@
       </c>
       <c r="L50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Finnish law obliges the funder to address research security while preserving researchers' freedom to choose topics.</t>
+          <t xml:space="preserve">The note sets out concrete proposals for clarifying how civil, dual-use and defence R&amp;I are positioned in EU programmes.</t>
         </is>
       </c>
       <c r="M50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Shapes how universities can participate in EU defence-adjacent research funding.</t>
         </is>
       </c>
       <c r="N50" s="3" t="inlineStr">
@@ -24531,12 +24531,12 @@
       </c>
       <c r="R50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research Council of Finland</t>
+          <t xml:space="preserve">CESAER</t>
         </is>
       </c>
       <c r="S50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.aka.fi/en/from-research-to-society/responsible-science/research-security/</t>
+          <t xml:space="preserve">https://www.cesaer.org/publications/clarifying-and-optimising-civil-dual-use-and-defence-research-and-innovation-in-future-eu-funding-programmes/</t>
         </is>
       </c>
     </row>
@@ -24546,12 +24546,12 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Self-assessment of research security</t>
+          <t xml:space="preserve">Research security</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-21</t>
+          <t xml:space="preserve">2026-08-19</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -24596,12 +24596,12 @@
       </c>
       <c r="L51" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Applications must include a research security appendix; inadequate risk assessment can make an application inadmissible or rejected.</t>
+          <t xml:space="preserve">Finnish law obliges the funder to address research security while preserving researchers' freedom to choose topics.</t>
         </is>
       </c>
       <c r="M51" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Turns research security from guidance into a funding eligibility condition.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="N51" s="3" t="inlineStr">
@@ -24631,7 +24631,7 @@
       </c>
       <c r="S51" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.aka.fi/en/research-funding/apply-for-funding/how-to-apply-for-funding/az-index-of-application-guidelines/research-security/</t>
+          <t xml:space="preserve">https://www.aka.fi/en/from-research-to-society/responsible-science/research-security/</t>
         </is>
       </c>
     </row>
@@ -24641,17 +24641,17 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Strategic by design: Making EU development cooperation work for critical raw materials - HCSS</t>
+          <t xml:space="preserve">Self-assessment of research security</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-08-21</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Hague Centre for Strategic Studies</t>
+          <t xml:space="preserve">Research Council of Finland</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
@@ -24676,7 +24676,7 @@
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Critical raw materials × R&amp;I / technology</t>
+          <t xml:space="preserve">Research security / dual use</t>
         </is>
       </c>
       <c r="J52" s="3" t="inlineStr">
@@ -24686,17 +24686,17 @@
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Research security / dual use</t>
         </is>
       </c>
       <c r="L52" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCSS finds EU critical-raw-material partnerships often struggle to convert political agreements into financeable projects.</t>
+          <t xml:space="preserve">Applications must include a research security appendix; inadequate risk assessment can make an application inadmissible or rejected.</t>
         </is>
       </c>
       <c r="M52" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Development-cooperation tools could help close feasibility, governance and financing gaps.</t>
+          <t xml:space="preserve">Turns research security from guidance into a funding eligibility condition.</t>
         </is>
       </c>
       <c r="N52" s="3" t="inlineStr">
@@ -24721,12 +24721,12 @@
       </c>
       <c r="R52" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Hague Centre for Strategic Studies</t>
+          <t xml:space="preserve">Research Council of Finland</t>
         </is>
       </c>
       <c r="S52" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://hcss.nl/wp-content/uploads/2026/08/Strategic-by-design-HCSS-2026-1.pdf</t>
+          <t xml:space="preserve">https://www.aka.fi/en/research-funding/apply-for-funding/how-to-apply-for-funding/az-index-of-application-guidelines/research-security/</t>
         </is>
       </c>
     </row>
@@ -24736,17 +24736,17 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research security as part of funding applications ‒ experiences and lessons from the first application round</t>
+          <t xml:space="preserve">Strategic by design: Making EU development cooperation work for critical raw materials - HCSS</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-21</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research Council of Finland</t>
+          <t xml:space="preserve">The Hague Centre for Strategic Studies</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
@@ -24771,7 +24771,7 @@
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research security / dual use</t>
+          <t xml:space="preserve">Critical raw materials × R&amp;I / technology</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
@@ -24781,17 +24781,17 @@
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Research security / dual use</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology</t>
         </is>
       </c>
       <c r="L53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Research Council of Finland reports requiring research-security self-assessment in Academy Project and Fellowship calls.</t>
+          <t xml:space="preserve">HCSS finds EU critical-raw-material partnerships often struggle to convert political agreements into financeable projects.</t>
         </is>
       </c>
       <c r="M53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Application requirements change how research-security risks are considered before public funding is awarded.</t>
+          <t xml:space="preserve">Development-cooperation tools could help close feasibility, governance and financing gaps.</t>
         </is>
       </c>
       <c r="N53" s="3" t="inlineStr">
@@ -24816,12 +24816,12 @@
       </c>
       <c r="R53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research Council of Finland</t>
+          <t xml:space="preserve">The Hague Centre for Strategic Studies</t>
         </is>
       </c>
       <c r="S53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.aka.fi/en/about-the-rcf/whats-new/blog2/2026/research-security-as-part-of-funding-applications--experiences-and-lessons-from-the-first-application-round/</t>
+          <t xml:space="preserve">https://hcss.nl/wp-content/uploads/2026/08/Strategic-by-design-HCSS-2026-1.pdf</t>
         </is>
       </c>
     </row>
@@ -24831,27 +24831,27 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exclusive: Commission offers three options for cutting back Horizon Europe industrial partnerships</t>
+          <t xml:space="preserve">Research security as part of funding applications ‒ experiences and lessons from the first application round</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-28T21:34Z</t>
+          <t xml:space="preserve">2026-09-21</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Science|Business</t>
+          <t xml:space="preserve">Research Council of Finland</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main C</t>
+          <t xml:space="preserve">Main A</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
@@ -24866,27 +24866,27 @@
       </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Research security / dual use</t>
         </is>
       </c>
       <c r="J54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business / industry</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Research security / dual use</t>
         </is>
       </c>
       <c r="L54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Commission presented options to consolidate Horizon Europe industrial partnerships from 60 to as few as 18.</t>
+          <t xml:space="preserve">The Research Council of Finland reports requiring research-security self-assessment in Academy Project and Fellowship calls.</t>
         </is>
       </c>
       <c r="M54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The proposal would materially reshape EU industry-research co-programming and funding structures.</t>
+          <t xml:space="preserve">Application requirements change how research-security risks are considered before public funding is awarded.</t>
         </is>
       </c>
       <c r="N54" s="3" t="inlineStr">
@@ -24911,12 +24911,12 @@
       </c>
       <c r="R54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Research Council of Finland</t>
         </is>
       </c>
       <c r="S54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMixgFBVV95cUxOemNUSndfajJncHdmLWRpbTZzOGFsYl8zZ09Sd0d2b0hXMDBUZ2pGaFFvVWhpWnpYaXhOUjdEbkJEeUJVZlU4bEZ1Sjl2azl5dmxOb0JkTkdUNDkwSk5KVThCVVJlU0xSVHJ1OGRpNFlLTUdyT3FVWnN2bkpZNWF1emhFQ3lTNVM5VXR0dVRBa2lOTmJmeHM4TUQ0UlliVmRJX1BoY2Nmcl8tWkJBMElRUHd3R1o3NXN0cmQxay1KRXVQa25tbHc?oc=5</t>
+          <t xml:space="preserve">https://www.aka.fi/en/about-the-rcf/whats-new/blog2/2026/research-security-as-part-of-funding-applications--experiences-and-lessons-from-the-first-application-round/</t>
         </is>
       </c>
     </row>
@@ -24926,12 +24926,12 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data Corner: Number of collaborative grants falls sharply in Horizon Europe</t>
+          <t xml:space="preserve">Exclusive: Commission offers three options for cutting back Horizon Europe industrial partnerships</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20T08:01Z</t>
+          <t xml:space="preserve">2026-09-28T21:34Z</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -24966,7 +24966,7 @@
       </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Business / industry</t>
         </is>
       </c>
       <c r="K55" s="3" t="inlineStr">
@@ -24976,12 +24976,12 @@
       </c>
       <c r="L55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Science|Business computes 5,271 collaborative Pillar 2 projects and EUR 32.9 billion from the European Commission dashboard in the first two-thirds</t>
+          <t xml:space="preserve">The Commission presented options to consolidate Horizon Europe industrial partnerships from 60 to as few as 18.</t>
         </is>
       </c>
       <c r="M55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">The proposal would materially reshape EU industry-research co-programming and funding structures.</t>
         </is>
       </c>
       <c r="N55" s="3" t="inlineStr">
@@ -25011,7 +25011,7 @@
       </c>
       <c r="S55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMixwFBVV95cUxPMXlLMlNkWGlnbXo3RVhONHpXeWp5N1hjaVNrajdNazRud1FHcW9nN3N3TVFUS3pEaHlaMHJIQ21ING9NUXZxbjNUYnJNb2d5UHg1Y0VNT1RhR3Ntc0tJQVlYeWZXT1BhU1k0YVdCcmNRejkybzZnei1zRjRLRXBBZ2RUWm5aakJZNGVrb2hBcm9BTXFUaUFHd2JhdS1vT2hMWG1QN2YwZHV3SnBXQ3RlT000VzY2bHdxejhFMFhmcGMyREl5NE1j?oc=5</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMixgFBVV95cUxOemNUSndfajJncHdmLWRpbTZzOGFsYl8zZ09Sd0d2b0hXMDBUZ2pGaFFvVWhpWnpYaXhOUjdEbkJEeUJVZlU4bEZ1Sjl2azl5dmxOb0JkTkdUNDkwSk5KVThCVVJlU0xSVHJ1OGRpNFlLTUdyT3FVWnN2bkpZNWF1emhFQ3lTNVM5VXR0dVRBa2lOTmJmeHM4TUQ0UlliVmRJX1BoY2Nmcl8tWkJBMElRUHd3R1o3NXN0cmQxay1KRXVQa25tbHc?oc=5</t>
         </is>
       </c>
     </row>
@@ -25021,17 +25021,17 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Critical Raw Materials: securing Europe’s supply and strategic autonomy | Atualidade | Parlamento Europeu</t>
+          <t xml:space="preserve">Data Corner: Number of collaborative grants falls sharply in Horizon Europe</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20T11:00Z</t>
+          <t xml:space="preserve">2026-10-20T08:01Z</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">European Parliament</t>
+          <t xml:space="preserve">Science|Business</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
@@ -25056,7 +25056,7 @@
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Critical raw materials × R&amp;I / technology</t>
+          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="J56" s="3" t="inlineStr">
@@ -25066,17 +25066,17 @@
       </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L56" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">European Parliament endorsed draft critical-raw-materials reforms, voting 470 to 83 with 108 abstentions.</t>
+          <t xml:space="preserve">Science|Business computes 5,271 collaborative Pillar 2 projects and EUR 32.9 billion from the European Commission dashboard in the first two-thirds</t>
         </is>
       </c>
       <c r="M56" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Concrete EU industrial technology-input policy reform with a direct innovation and supply-security connection.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="N56" s="3" t="inlineStr">
@@ -25106,77 +25106,77 @@
       </c>
       <c r="S56" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMi0wFBVV95cUxNTlFrR1R3UDM5NzFXdnpldWQtVzhUZ1Y4NnZDMmhmN0g4ZjdZWFJDVy1xRDNtbWtyYVBmV1BCaHZDcWpJbFdrT0xtbzA1Q1pqS1V6Uy1tdUFBUkxHS2ttQjlGVlRib3ZtTU50RHZ0R3o3ZGZteWlqbldkeVRpSEhNYWt6NWFJRVR6dTA2dVpHb2JFbXM0Zk5Sb2l1UExZZi1yQUlST3ptVEVhSE5CZFg5M2FLZTBVVTFUaUQ4VUlULWxkbVhhX3o3am5rbUhIRTdncE1F?oc=5</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMixwFBVV95cUxPMXlLMlNkWGlnbXo3RVhONHpXeWp5N1hjaVNrajdNazRud1FHcW9nN3N3TVFUS3pEaHlaMHJIQ21ING9NUXZxbjNUYnJNb2d5UHg1Y0VNT1RhR3Ntc0tJQVlYeWZXT1BhU1k0YVdCcmNRejkybzZnei1zRjRLRXBBZ2RUWm5aakJZNGVrb2hBcm9BTXFUaUFHd2JhdS1vT2hMWG1QN2YwZHV3SnBXQ3RlT000VzY2bHdxejhFMFhmcGMyREl5NE1j?oc=5</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Statement by European Research Institute Directors</t>
+          <t xml:space="preserve">Critical Raw Materials: securing Europe’s supply and strategic autonomy | Atualidade | Parlamento Europeu</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2021-03-22</t>
+          <t xml:space="preserve">2026-10-20T11:00Z</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWP</t>
+          <t xml:space="preserve">European Parliament</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historical</t>
+          <t xml:space="preserve">Main C</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">China</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asia &amp; Pacific</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research security / dual use</t>
+          <t xml:space="preserve">Critical raw materials × R&amp;I / technology</t>
         </is>
       </c>
       <c r="J57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Universities / research institutions</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: China; issue: Research security / dual use</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology</t>
         </is>
       </c>
       <c r="L57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Same joint statement as the FIIA record, published by SWP, protesting Chinese sanctions on European researchers.</t>
+          <t xml:space="preserve">European Parliament endorsed draft critical-raw-materials reforms, voting 470 to 83 with 108 abstentions.</t>
         </is>
       </c>
       <c r="M57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Duplicate publication across signatories risks counting one statement twice in the corpus.</t>
+          <t xml:space="preserve">Concrete EU industrial technology-input policy reform with a direct innovation and supply-security connection.</t>
         </is>
       </c>
       <c r="N57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">review</t>
+          <t xml:space="preserve">keep</t>
         </is>
       </c>
       <c r="O57" s="3" t="inlineStr">
@@ -25186,12 +25186,12 @@
       </c>
       <c r="P57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-16T11:09:09Z</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="Q57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">worker-b-20260916T103241Z-d69fa410f5f1</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="R57" s="3" t="inlineStr">
@@ -25201,7 +25201,7 @@
       </c>
       <c r="S57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.swp-berlin.org/presse/detail/statement-by-european-research-institute-directors</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMi0wFBVV95cUxNTlFrR1R3UDM5NzFXdnpldWQtVzhUZ1Y4NnZDMmhmN0g4ZjdZWFJDVy1xRDNtbWtyYVBmV1BCaHZDcWpJbFdrT0xtbzA1Q1pqS1V6Uy1tdUFBUkxHS2ttQjlGVlRib3ZtTU50RHZ0R3o3ZGZteWlqbldkeVRpSEhNYWt6NWFJRVR6dTA2dVpHb2JFbXM0Zk5Sb2l1UExZZi1yQUlST3ptVEVhSE5CZFg5M2FLZTBVVTFUaUQ4VUlULWxkbVhhX3o3am5rbUhIRTdncE1F?oc=5</t>
         </is>
       </c>
     </row>
@@ -25211,22 +25211,22 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sustainable productivity growth in agriculture: The role of shifts in R&amp;D investments and technology</t>
+          <t xml:space="preserve">Statement by European Research Institute Directors</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-04-07</t>
+          <t xml:space="preserve">2021-03-22</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Applied Economic Perspectives and Policy (Wiley)</t>
+          <t xml:space="preserve">SWP</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main A</t>
+          <t xml:space="preserve">Historical</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
@@ -25236,42 +25236,42 @@
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brazil; China; India</t>
+          <t xml:space="preserve">China</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Americas; Asia &amp; Pacific</t>
+          <t xml:space="preserve">Asia &amp; Pacific</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">China in Africa / LAC</t>
+          <t xml:space="preserve">Research security / dual use</t>
         </is>
       </c>
       <c r="J58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Universities / research institutions</t>
         </is>
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: Brazil, China, India; issue: China in Africa / LAC</t>
+          <t xml:space="preserve">Region: China; issue: Research security / dual use</t>
         </is>
       </c>
       <c r="L58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modelling suggests shifting research from yield maximisation to input saving could cut chemical use substantially.</t>
+          <t xml:space="preserve">Same joint statement as the FIIA record, published by SWP, protesting Chinese sanctions on European researchers.</t>
         </is>
       </c>
       <c r="M58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Duplicate publication across signatories risks counting one statement twice in the corpus.</t>
         </is>
       </c>
       <c r="N58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">keep</t>
+          <t xml:space="preserve">review</t>
         </is>
       </c>
       <c r="O58" s="3" t="inlineStr">
@@ -25281,22 +25281,22 @@
       </c>
       <c r="P58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">2026-09-16T11:09:09Z</t>
         </is>
       </c>
       <c r="Q58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">worker-b-20260916T103241Z-d69fa410f5f1</t>
         </is>
       </c>
       <c r="R58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zuzana Smeets Křístková; Michiel van Dijk; Robert M'Barek; Hans van Meijl; Tomas Ratinger</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="S58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://publications.jrc.ec.europa.eu/repository/handle/JRC142267</t>
+          <t xml:space="preserve">https://www.swp-berlin.org/presse/detail/statement-by-european-research-institute-directors</t>
         </is>
       </c>
     </row>
@@ -25306,17 +25306,17 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Report shows country participation in European Innovation Ecosystems Programme</t>
+          <t xml:space="preserve">Sustainable productivity growth in agriculture: The role of shifts in R&amp;D investments and technology</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-04-22</t>
+          <t xml:space="preserve">2026-04-07</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ERA Portal Austria</t>
+          <t xml:space="preserve">Applied Economic Perspectives and Policy (Wiley)</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
@@ -25331,17 +25331,17 @@
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ukraine</t>
+          <t xml:space="preserve">Brazil; China; India</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Europe — enlargement</t>
+          <t xml:space="preserve">Americas; Asia &amp; Pacific</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">China in Africa / LAC</t>
         </is>
       </c>
       <c r="J59" s="3" t="inlineStr">
@@ -25351,17 +25351,17 @@
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: Ukraine; issue: EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: Brazil, China, India; issue: China in Africa / LAC</t>
         </is>
       </c>
       <c r="L59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The report compares country participation in European Innovation Ecosystems.</t>
+          <t xml:space="preserve">Modelling suggests shifting research from yield maximisation to input saving could cut chemical use substantially.</t>
         </is>
       </c>
       <c r="M59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Participation patterns reveal uneven engagement across national innovation ecosystems.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="N59" s="3" t="inlineStr">
@@ -25386,12 +25386,12 @@
       </c>
       <c r="R59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ERA Portal Austria</t>
+          <t xml:space="preserve">Zuzana Smeets Křístková; Michiel van Dijk; Robert M'Barek; Hans van Meijl; Tomas Ratinger</t>
         </is>
       </c>
       <c r="S59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://era.gv.at/news-items/report-shows-country-participation-in-european-innovation-ecosystems-programme/</t>
+          <t xml:space="preserve">https://publications.jrc.ec.europa.eu/repository/handle/JRC142267</t>
         </is>
       </c>
     </row>
@@ -25401,17 +25401,17 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overcoming legal barriers for the uptake of innovation procurement in the EU</t>
+          <t xml:space="preserve">Report shows country participation in European Innovation Ecosystems Programme</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-05-22</t>
+          <t xml:space="preserve">2026-04-22</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Publications Office of the European Union</t>
+          <t xml:space="preserve">ERA Portal Austria</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
@@ -25426,12 +25426,12 @@
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">United States; Canada; China</t>
+          <t xml:space="preserve">Ukraine</t>
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Americas; Asia &amp; Pacific</t>
+          <t xml:space="preserve">Europe — enlargement</t>
         </is>
       </c>
       <c r="I60" s="3" t="inlineStr">
@@ -25446,17 +25446,17 @@
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: United States, Canada, China; issue: EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: Ukraine; issue: EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L60" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Report finds European innovation procurement lags other major economies and blames weak incentives in EU law.</t>
+          <t xml:space="preserve">The report compares country participation in European Innovation Ecosystems.</t>
         </is>
       </c>
       <c r="M60" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Participation patterns reveal uneven engagement across national innovation ecosystems.</t>
         </is>
       </c>
       <c r="N60" s="3" t="inlineStr">
@@ -25481,12 +25481,12 @@
       </c>
       <c r="R60" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Directorate-General for Research and Innovation (European Commission); Corvers Procurement Services</t>
+          <t xml:space="preserve">ERA Portal Austria</t>
         </is>
       </c>
       <c r="S60" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://era.gv.at/news-items/new-report-urges-stronger-eu-rules-to-boost-innovation-procurement/</t>
+          <t xml:space="preserve">https://era.gv.at/news-items/report-shows-country-participation-in-european-innovation-ecosystems-programme/</t>
         </is>
       </c>
     </row>
@@ -25496,17 +25496,17 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Europe has produced tech champions: Here is what they can teach us</t>
+          <t xml:space="preserve">Overcoming legal barriers for the uptake of innovation procurement in the EU</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-05-27</t>
+          <t xml:space="preserve">2026-05-22</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Centre for European Reform</t>
+          <t xml:space="preserve">Publications Office of the European Union</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
@@ -25521,12 +25521,12 @@
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">China</t>
+          <t xml:space="preserve">United States; Canada; China</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asia &amp; Pacific</t>
+          <t xml:space="preserve">Americas; Asia &amp; Pacific</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr">
@@ -25536,22 +25536,22 @@
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business / industry</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: China; issue: EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: United States, Canada, China; issue: EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Europe has produced genuine tech leaders whose experience should shape competitiveness and innovation policy.</t>
+          <t xml:space="preserve">Report finds European innovation procurement lags other major economies and blames weak incentives in EU law.</t>
         </is>
       </c>
       <c r="M61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shifts the policy debate from Europe's missing giants to what its successes actually required.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="N61" s="3" t="inlineStr">
@@ -25576,12 +25576,12 @@
       </c>
       <c r="R61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">James Green</t>
+          <t xml:space="preserve">Directorate-General for Research and Innovation (European Commission); Corvers Procurement Services</t>
         </is>
       </c>
       <c r="S61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.cer.eu/sites/default/files/JG_tech_success_27.5.26.pdf</t>
+          <t xml:space="preserve">https://era.gv.at/news-items/new-report-urges-stronger-eu-rules-to-boost-innovation-procurement/</t>
         </is>
       </c>
     </row>
@@ -25591,17 +25591,17 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tracking country innovation performance: The Innovation Output Indicator 2025</t>
+          <t xml:space="preserve">Europe has produced tech champions: Here is what they can teach us</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-01</t>
+          <t xml:space="preserve">2026-05-27</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">JRC Publications Repository</t>
+          <t xml:space="preserve">Centre for European Reform</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
@@ -25631,7 +25631,7 @@
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Business / industry</t>
         </is>
       </c>
       <c r="K62" s="3" t="inlineStr">
@@ -25641,12 +25641,12 @@
       </c>
       <c r="L62" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sweden, Ireland and Germany lead the EU; the EU trails the US, Korea and Japan but beats China.</t>
+          <t xml:space="preserve">Europe has produced genuine tech leaders whose experience should shape competitiveness and innovation policy.</t>
         </is>
       </c>
       <c r="M62" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The indicator feeds DG RTD monitoring of Framework Programme objectives and complements the European Innovation Scoreboard.</t>
+          <t xml:space="preserve">Shifts the policy debate from Europe's missing giants to what its successes actually required.</t>
         </is>
       </c>
       <c r="N62" s="3" t="inlineStr">
@@ -25671,12 +25671,12 @@
       </c>
       <c r="R62" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">BELLO, Michela, RAVANOS, Panagiotis, TESSARIN, Milene</t>
+          <t xml:space="preserve">James Green</t>
         </is>
       </c>
       <c r="S62" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://publications.jrc.ec.europa.eu/repository/handle/JRC145507</t>
+          <t xml:space="preserve">https://www.cer.eu/sites/default/files/JG_tech_success_27.5.26.pdf</t>
         </is>
       </c>
     </row>
@@ -25686,17 +25686,17 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mapping of technology specialisation, complexity and relatedness of the EU and selected global partners</t>
+          <t xml:space="preserve">Tracking country innovation performance: The Innovation Output Indicator 2025</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-02</t>
+          <t xml:space="preserve">2026-06-01</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">CEPS</t>
+          <t xml:space="preserve">JRC Publications Repository</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
@@ -25736,12 +25736,12 @@
       </c>
       <c r="L63" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The EU leads in scientific output but trails the US and China in patenting and venture capital.</t>
+          <t xml:space="preserve">Sweden, Ireland and Germany lead the EU; the EU trails the US, Korea and Japan but beats China.</t>
         </is>
       </c>
       <c r="M63" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quantifies the gap between European research strength and commercialisation across strategic technologies.</t>
+          <t xml:space="preserve">The indicator feeds DG RTD monitoring of Framework Programme objectives and complements the European Innovation Scoreboard.</t>
         </is>
       </c>
       <c r="N63" s="3" t="inlineStr">
@@ -25766,12 +25766,12 @@
       </c>
       <c r="R63" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pierre-Alexandre Balland, Andrea Renda</t>
+          <t xml:space="preserve">BELLO, Michela, RAVANOS, Panagiotis, TESSARIN, Milene</t>
         </is>
       </c>
       <c r="S63" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://cdn.ceps.eu/wp-content/uploads/2024/09/Code-of-Conduct-CEPS-events.pdf</t>
+          <t xml:space="preserve">https://publications.jrc.ec.europa.eu/repository/handle/JRC145507</t>
         </is>
       </c>
     </row>
@@ -25781,37 +25781,37 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Is Germany benefitting yet from the crisis in US research?</t>
+          <t xml:space="preserve">Mapping of technology specialisation, complexity and relatedness of the EU and selected global partners</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-27T07:00Z</t>
+          <t xml:space="preserve">2026-06-02</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Science|Business</t>
+          <t xml:space="preserve">CEPS</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main C</t>
+          <t xml:space="preserve">Main A</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">United States</t>
+          <t xml:space="preserve">China</t>
         </is>
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Americas</t>
+          <t xml:space="preserve">Asia &amp; Pacific</t>
         </is>
       </c>
       <c r="I64" s="3" t="inlineStr">
@@ -25821,22 +25821,22 @@
       </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Universities / research institutions</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: United States; issue: EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: China; issue: EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L64" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">US research uncertainty is increasing interest in German academic jobs and recruitment initiatives.</t>
+          <t xml:space="preserve">The EU leads in scientific output but trails the US and China in patenting and venture capital.</t>
         </is>
       </c>
       <c r="M64" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The shift may strengthen German talent inflows, though structural career barriers remain.</t>
+          <t xml:space="preserve">Quantifies the gap between European research strength and commercialisation across strategic technologies.</t>
         </is>
       </c>
       <c r="N64" s="3" t="inlineStr">
@@ -25861,12 +25861,12 @@
       </c>
       <c r="R64" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Pierre-Alexandre Balland, Andrea Renda</t>
         </is>
       </c>
       <c r="S64" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMiiwFBVV95cUxPZ0ZrOUpoVzRmZ2ptUndxRVpyTjk0djJiMlJCZzlTT0sxSmo0WnBRQUxtTl90TktnQTg0T0xGd1lGOURyRjNZd18wWklidU5OdVBkRUtfWmUtX084Vkd6dU16MExzVzlEVDNfTm5YSGZPTWNBYnF5QzNFYUhRb0JBLWdsVnhDWUVaWU5R?oc=5</t>
+          <t xml:space="preserve">https://cdn.ceps.eu/wp-content/uploads/2024/09/Code-of-Conduct-CEPS-events.pdf</t>
         </is>
       </c>
     </row>
@@ -25876,17 +25876,17 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Europe must tighten grip on AI supply chain, experts warn</t>
+          <t xml:space="preserve">Is Germany benefitting yet from the crisis in US research?</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14T02:03Z</t>
+          <t xml:space="preserve">2026-08-27T07:00Z</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Euractiv</t>
+          <t xml:space="preserve">Science|Business</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
@@ -25901,37 +25901,37 @@
       </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">China</t>
+          <t xml:space="preserve">United States</t>
         </is>
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asia &amp; Pacific</t>
+          <t xml:space="preserve">Americas</t>
         </is>
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU-facing technology standards / regulatory alignment</t>
+          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Universities / research institutions</t>
         </is>
       </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: China; issue: EU-facing technology standards / regulatory alignment</t>
+          <t xml:space="preserve">Region: United States; issue: EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L65" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A new expert report urged Europe to expand compute capacity and reduce strategic AI supply-chain dependencies.</t>
+          <t xml:space="preserve">US research uncertainty is increasing interest in German academic jobs and recruitment initiatives.</t>
         </is>
       </c>
       <c r="M65" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compute ownership and supply-chain control affect Europe’s ability to develop and deploy advanced AI independently.</t>
+          <t xml:space="preserve">The shift may strengthen German talent inflows, though structural career barriers remain.</t>
         </is>
       </c>
       <c r="N65" s="3" t="inlineStr">
@@ -25961,27 +25961,27 @@
       </c>
       <c r="S65" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMikAFBVV95cUxPZEV0SmRDTGhaSkh2MnBPTjBsWjh4VGpLWGFESlYwSklXUUxBVkhIMXdDZGNaR2hZVFE1VXVxV0Q2VlJwYjV0alVxRnVpeERjY3NEMmZkNm91Tk5BYW1QU05DVmpyNGM1ZkN4aUlCLXFzbWNHUHZIZWw4a3V1OVA3cElQQWo2dGRBSzYwZW1DQXo?oc=5</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMiiwFBVV95cUxPZ0ZrOUpoVzRmZ2ptUndxRVpyTjk0djJiMlJCZzlTT0sxSmo0WnBRQUxtTl90TktnQTg0T0xGd1lGOURyRjNZd18wWklidU5OdVBkRUtfWmUtX084Vkd6dU16MExzVzlEVDNfTm5YSGZPTWNBYnF5QzNFYUhRb0JBLWdsVnhDWUVaWU5R?oc=5</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU-China research cooperation limited to ‘targeted areas’</t>
+          <t xml:space="preserve">Europe must tighten grip on AI supply chain, experts warn</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-10T07:00Z</t>
+          <t xml:space="preserve">2026-09-14T02:03Z</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research Professional News</t>
+          <t xml:space="preserve">Euractiv</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
@@ -26006,7 +26006,7 @@
       </c>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transnational R&amp;I and innovation policy</t>
+          <t xml:space="preserve">EU-facing technology standards / regulatory alignment</t>
         </is>
       </c>
       <c r="J66" s="3" t="inlineStr">
@@ -26016,22 +26016,22 @@
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: China; issue: Transnational R&amp;I and innovation policy</t>
+          <t xml:space="preserve">Region: China; issue: EU-facing technology standards / regulatory alignment</t>
         </is>
       </c>
       <c r="L66" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">A new expert report urged Europe to expand compute capacity and reduce strategic AI supply-chain dependencies.</t>
         </is>
       </c>
       <c r="M66" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">This may shift the risk–reward balance of EU–China research, technology and innovation cooperation.</t>
+          <t xml:space="preserve">Compute ownership and supply-chain control affect Europe’s ability to develop and deploy advanced AI independently.</t>
         </is>
       </c>
       <c r="N66" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">provisional</t>
+          <t xml:space="preserve">keep</t>
         </is>
       </c>
       <c r="O66" s="3" t="inlineStr">
@@ -26056,7 +26056,7 @@
       </c>
       <c r="S66" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMixwFBVV95cUxQR1JiOFNtQlZBYUJUUThOYXVYSjFad2h0TG5OSm9ZdDBaY0NrbVk3UkkxUlZJMWFPczJySWd5RmwtYmZsdFE2bS1iOGJnMHFacHBtWE5GUWpqRTN3QXR4SHVtdE1ZRktGY3V6SUc0OWtIQVhSMUp5QVk2ZjE0N29TdFp6ZzgwTmx0aXpkMFpsM2lfb2xrWUtyWXJLY1hlYnRqNEhQWHNZLUhZZThpeklQU3NHWXQ2SGZhNkpmTllLU1JCN1NMU2Jv?oc=5</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMikAFBVV95cUxPZEV0SmRDTGhaSkh2MnBPTjBsWjh4VGpLWGFESlYwSklXUUxBVkhIMXdDZGNaR2hZVFE1VXVxV0Q2VlJwYjV0alVxRnVpeERjY3NEMmZkNm91Tk5BYW1QU05DVmpyNGM1ZkN4aUlCLXFzbWNHUHZIZWw4a3V1OVA3cElQQWo2dGRBSzYwZW1DQXo?oc=5</t>
         </is>
       </c>
     </row>
@@ -26066,17 +26066,17 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The 17th EU-China Joint Steering Committee meeting on Science and Technology Cooperation - European Commission</t>
+          <t xml:space="preserve">EU-China research cooperation limited to ‘targeted areas’</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-13T14:31Z</t>
+          <t xml:space="preserve">2026-08-10T07:00Z</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU Research &amp; Innovation</t>
+          <t xml:space="preserve">Research Professional News</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
@@ -26116,17 +26116,17 @@
       </c>
       <c r="L67" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The EU and China held their 17th science-and-technology committee meeting, assessing shared research flagships and priorities.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="M67" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The meeting directly concerns joint research frameworks, researcher mobility and cross-border science cooperation.</t>
+          <t xml:space="preserve">This may shift the risk–reward balance of EU–China research, technology and innovation cooperation.</t>
         </is>
       </c>
       <c r="N67" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">keep</t>
+          <t xml:space="preserve">provisional</t>
         </is>
       </c>
       <c r="O67" s="3" t="inlineStr">
@@ -26151,7 +26151,7 @@
       </c>
       <c r="S67" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMiigJBVV95cUxNbndpTU9lc2hONXNPa2pCMm54Y05ZV1hCcm5BMTUyQ19sRTV4S1lkTGlyZlVNRFRMd2lWS3E3WWdRZ28tOUlXbFVsRU5nTFFvT2xISW8zOWZtSF81R1prcHJVbGVEZFY5YXdpRmxHcG5WT0VkZ2dYYWI0SWdqVVo4YWh4VVdfNkdQdFlTNjk0enltWENEZF92UHRicEhjS1dVNGtZRzhrQ20zQ1l4M0Eyc21kck9JREJzR0ZCTXNlN0FnaDk3NXRoLW1kLWU2Wlc3T1lGcEZ5V09NSzBJSGNYR2RFbWstSERDSm9YVXpSdXZKT1ByUkdsZXdnV3UwR0NwdVRIT3AzY1FGdw?oc=5</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMixwFBVV95cUxQR1JiOFNtQlZBYUJUUThOYXVYSjFad2h0TG5OSm9ZdDBaY0NrbVk3UkkxUlZJMWFPczJySWd5RmwtYmZsdFE2bS1iOGJnMHFacHBtWE5GUWpqRTN3QXR4SHVtdE1ZRktGY3V6SUc0OWtIQVhSMUp5QVk2ZjE0N29TdFp6ZzgwTmx0aXpkMFpsM2lfb2xrWUtyWXJLY1hlYnRqNEhQWHNZLUhZZThpeklQU3NHWXQ2SGZhNkpmTllLU1JCN1NMU2Jv?oc=5</t>
         </is>
       </c>
     </row>
@@ -26161,17 +26161,17 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Science Europe publishes response to EC consultation on evaluation of the dual-use regulation</t>
+          <t xml:space="preserve">The 17th EU-China Joint Steering Committee meeting on Science and Technology Cooperation - European Commission</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-15</t>
+          <t xml:space="preserve">2026-10-13T14:31Z</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ERA Portal Austria</t>
+          <t xml:space="preserve">EU Research &amp; Innovation</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
@@ -26186,17 +26186,17 @@
       </c>
       <c r="G68" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">China</t>
         </is>
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Asia &amp; Pacific</t>
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research security / dual use; Transnational R&amp;I and innovation policy</t>
+          <t xml:space="preserve">Transnational R&amp;I and innovation policy</t>
         </is>
       </c>
       <c r="J68" s="3" t="inlineStr">
@@ -26206,17 +26206,17 @@
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Research security / dual use, Transnational R&amp;I and innovation policy</t>
+          <t xml:space="preserve">Region: China; issue: Transnational R&amp;I and innovation policy</t>
         </is>
       </c>
       <c r="L68" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Science Europe issued an October 2026 response to an EU consultation on dual-use controls and research cooperation.</t>
+          <t xml:space="preserve">The EU and China held their 17th science-and-technology committee meeting, assessing shared research flagships and priorities.</t>
         </is>
       </c>
       <c r="M68" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dual-use guidance can affect researchers’ international collaboration and compliance burdens.</t>
+          <t xml:space="preserve">The meeting directly concerns joint research frameworks, researcher mobility and cross-border science cooperation.</t>
         </is>
       </c>
       <c r="N68" s="3" t="inlineStr">
@@ -26241,12 +26241,12 @@
       </c>
       <c r="R68" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ERA Portal Austria</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="S68" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://era.gv.at/news-items/science-europe-publishes-response-to-ec-consultation-on-evaluation-of-the-dual-use-regulation/</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMiigJBVV95cUxNbndpTU9lc2hONXNPa2pCMm54Y05ZV1hCcm5BMTUyQ19sRTV4S1lkTGlyZlVNRFRMd2lWS3E3WWdRZ28tOUlXbFVsRU5nTFFvT2xISW8zOWZtSF81R1prcHJVbGVEZFY5YXdpRmxHcG5WT0VkZ2dYYWI0SWdqVVo4YWh4VVdfNkdQdFlTNjk0enltWENEZF92UHRicEhjS1dVNGtZRzhrQ20zQ1l4M0Eyc21kck9JREJzR0ZCTXNlN0FnaDk3NXRoLW1kLWU2Wlc3T1lGcEZ5V09NSzBJSGNYR2RFbWstSERDSm9YVXpSdXZKT1ByUkdsZXdnV3UwR0NwdVRIT3AzY1FGdw?oc=5</t>
         </is>
       </c>
     </row>
@@ -26256,27 +26256,27 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deep dive on critical raw materials for hydrogen technologies in the EU</t>
+          <t xml:space="preserve">Science Europe publishes response to EC consultation on evaluation of the dual-use regulation</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20</t>
+          <t xml:space="preserve">2026-10-15</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">JRC Publications Repository</t>
+          <t xml:space="preserve">ERA Portal Austria</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main A</t>
+          <t xml:space="preserve">Main C</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
@@ -26291,7 +26291,7 @@
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Critical raw materials × R&amp;I / technology; EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Research security / dual use; Transnational R&amp;I and innovation policy</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
@@ -26301,17 +26301,17 @@
       </c>
       <c r="K69" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology, EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Research security / dual use, Transnational R&amp;I and innovation policy</t>
         </is>
       </c>
       <c r="L69" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU JRC models 2030-2050 material-supply vulnerabilities for hydrogen technologies; iridium/platinum bottlenecks are scenario-based, not observations.</t>
+          <t xml:space="preserve">Science Europe issued an October 2026 response to an EU consultation on dual-use controls and research cooperation.</t>
         </is>
       </c>
       <c r="M69" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Dual-use guidance can affect researchers’ international collaboration and compliance burdens.</t>
         </is>
       </c>
       <c r="N69" s="3" t="inlineStr">
@@ -26336,32 +26336,32 @@
       </c>
       <c r="R69" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">BOLARD, Julien, NOHL, Markus, PAVEL, Claudiu, ISTRATE, Robert, EYNARD, Umberto, BLAGOEVA, Darina, DOLCI, Francesco, KUZOV, Teodor</t>
+          <t xml:space="preserve">ERA Portal Austria</t>
         </is>
       </c>
       <c r="S69" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://publications.jrc.ec.europa.eu/repository/handle/JRC148105</t>
+          <t xml:space="preserve">https://era.gv.at/news-items/science-europe-publishes-response-to-ec-consultation-on-evaluation-of-the-dual-use-regulation/</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Connecting European Science: ESF Joins Horizon Europe Initiatives to Streamline Research Infrastructure Access - ESF</t>
+          <t xml:space="preserve">Deep dive on critical raw materials for hydrogen technologies in the EU</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-10</t>
+          <t xml:space="preserve">2026-10-20</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">European Science Foundation</t>
+          <t xml:space="preserve">JRC Publications Repository</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
@@ -26386,27 +26386,27 @@
       </c>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Critical raw materials × R&amp;I / technology; EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business / industry</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology, EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L70" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Access2Access, FUND-RI and COORDINA-INNOV address facility access, sustainable funding and research-infrastructure collaboration with industry.</t>
+          <t xml:space="preserve">EU JRC models 2030-2050 material-supply vulnerabilities for hydrogen technologies; iridium/platinum bottlenecks are scenario-based, not observations.</t>
         </is>
       </c>
       <c r="M70" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Together they target structural fragmentation across Europe’s research-infrastructure ecosystem.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="N70" s="3" t="inlineStr">
@@ -26431,12 +26431,12 @@
       </c>
       <c r="R70" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ines AZAIEZ</t>
+          <t xml:space="preserve">BOLARD, Julien, NOHL, Markus, PAVEL, Claudiu, ISTRATE, Robert, EYNARD, Umberto, BLAGOEVA, Darina, DOLCI, Francesco, KUZOV, Teodor</t>
         </is>
       </c>
       <c r="S70" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.esf.org/esf-joins-horizon-europe-initiatives-to-streamline-research-infrastructure-access/</t>
+          <t xml:space="preserve">https://publications.jrc.ec.europa.eu/repository/handle/JRC148105</t>
         </is>
       </c>
     </row>
@@ -26446,27 +26446,27 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU research and innovation funding expands to defence and dual-use technologies</t>
+          <t xml:space="preserve">Connecting European Science: ESF Joins Horizon Europe Initiatives to Streamline Research Infrastructure Access - ESF</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-24</t>
+          <t xml:space="preserve">2026-06-10</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ERA Portal Austria</t>
+          <t xml:space="preserve">European Science Foundation</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main C</t>
+          <t xml:space="preserve">Main A</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
@@ -26481,27 +26481,27 @@
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research security / dual use</t>
+          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Business / industry</t>
         </is>
       </c>
       <c r="K71" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Research security / dual use</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L71" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The 2026 EIC programme now allows dual-use and defence applicants and adds a €100 million defence scale-up call.</t>
+          <t xml:space="preserve">Access2Access, FUND-RI and COORDINA-INNOV address facility access, sustainable funding and research-infrastructure collaboration with industry.</t>
         </is>
       </c>
       <c r="M71" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The amendment changes eligibility and financing channels, directly expanding EU support for strategic technology scale-up.</t>
+          <t xml:space="preserve">Together they target structural fragmentation across Europe’s research-infrastructure ecosystem.</t>
         </is>
       </c>
       <c r="N71" s="3" t="inlineStr">
@@ -26526,12 +26526,12 @@
       </c>
       <c r="R71" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ERA Portal Austria</t>
+          <t xml:space="preserve">Ines AZAIEZ</t>
         </is>
       </c>
       <c r="S71" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://era.gv.at/news-items/eu-research-and-innovation-funding-expands-to-defence-and-dual-use-technologies/</t>
+          <t xml:space="preserve">https://www.esf.org/esf-joins-horizon-europe-initiatives-to-streamline-research-infrastructure-access/</t>
         </is>
       </c>
     </row>
@@ -26541,12 +26541,12 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Guild urges safeguards as FP10 opens to dual-use research</t>
+          <t xml:space="preserve">EU research and innovation funding expands to defence and dual-use technologies</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-07-01</t>
+          <t xml:space="preserve">2026-06-24</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
@@ -26556,12 +26556,12 @@
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main A</t>
+          <t xml:space="preserve">Main C</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">
@@ -26581,7 +26581,7 @@
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Universities / research institutions</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K72" s="3" t="inlineStr">
@@ -26591,12 +26591,12 @@
       </c>
       <c r="L72" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Guild argues dual-use research needs targeted safeguards without weakening open frontier research.</t>
+          <t xml:space="preserve">The 2026 EIC programme now allows dual-use and defence applicants and adds a €100 million defence scale-up call.</t>
         </is>
       </c>
       <c r="M72" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Broad restrictions could damage basic research and international collaboration.</t>
+          <t xml:space="preserve">The amendment changes eligibility and financing channels, directly expanding EU support for strategic technology scale-up.</t>
         </is>
       </c>
       <c r="N72" s="3" t="inlineStr">
@@ -26626,7 +26626,7 @@
       </c>
       <c r="S72" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://era.gv.at/news-items/the-guild-urges-safeguards-as-fp10-opens-to-dual-use-research/</t>
+          <t xml:space="preserve">https://era.gv.at/news-items/eu-research-and-innovation-funding-expands-to-defence-and-dual-use-technologies/</t>
         </is>
       </c>
     </row>
@@ -26636,12 +26636,12 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">European Innovation Act should put universities at the heart of innovation, EUA says</t>
+          <t xml:space="preserve">The Guild urges safeguards as FP10 opens to dual-use research</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-07-06</t>
+          <t xml:space="preserve">2026-07-01</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -26671,27 +26671,27 @@
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Research security / dual use</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Universities / research institutions; Business / industry</t>
+          <t xml:space="preserve">Universities / research institutions</t>
         </is>
       </c>
       <c r="K73" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Research security / dual use</t>
         </is>
       </c>
       <c r="L73" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EUA argues the Act should build a shared European innovation culture with universities at its core.</t>
+          <t xml:space="preserve">The Guild argues dual-use research needs targeted safeguards without weakening open frontier research.</t>
         </is>
       </c>
       <c r="M73" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Act would be the first EU law focused solely on innovation.</t>
+          <t xml:space="preserve">Broad restrictions could damage basic research and international collaboration.</t>
         </is>
       </c>
       <c r="N73" s="3" t="inlineStr">
@@ -26721,7 +26721,7 @@
       </c>
       <c r="S73" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://era.gv.at/news-items/european-innovation-act-should-put-universities-at-the-heart-of-innovation-eua-says/</t>
+          <t xml:space="preserve">https://era.gv.at/news-items/the-guild-urges-safeguards-as-fp10-opens-to-dual-use-research/</t>
         </is>
       </c>
     </row>
@@ -26731,27 +26731,27 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU's cybersecurity agency granted access to Mythos 5 AI model, Commission says</t>
+          <t xml:space="preserve">European Innovation Act should put universities at the heart of innovation, EUA says</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-10T08:56Z</t>
+          <t xml:space="preserve">2026-07-06</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reuters</t>
+          <t xml:space="preserve">ERA Portal Austria</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main C</t>
+          <t xml:space="preserve">Main A</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
       <c r="G74" s="3" t="inlineStr">
@@ -26766,27 +26766,27 @@
       </c>
       <c r="I74" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU-facing technology standards / regulatory alignment</t>
+          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Universities / research institutions; Business / industry</t>
         </is>
       </c>
       <c r="K74" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: EU-facing technology standards / regulatory alignment</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L74" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The EU cybersecurity agency received access to leading AI models to assess cybersecurity implications.</t>
+          <t xml:space="preserve">EUA argues the Act should build a shared European innovation culture with universities at its core.</t>
         </is>
       </c>
       <c r="M74" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Direct model access enables independent security testing and evidence for European AI and cyber-risk governance.</t>
+          <t xml:space="preserve">The Act would be the first EU law focused solely on innovation.</t>
         </is>
       </c>
       <c r="N74" s="3" t="inlineStr">
@@ -26811,12 +26811,12 @@
       </c>
       <c r="R74" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ERA Portal Austria</t>
         </is>
       </c>
       <c r="S74" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMivAFBVV95cUxPRWVkQ1I1dzB2Wm10ZmloY0d5bW9PNEpSSnVTT0V5bHU0SXNsMnEyY1c0V2NmVnhzSm1qZ0JXZ1dsaHBDNkJmRXdzaWVaeks5ekhROVF0SjU3cGQ5VWRPc1NPRFd2UmtYRTJPZWVLamFvRjV0WmRnWk04UW13UUcwZnlGNFlORzd2cFUxZ056UkRJcEJaekZSMFM3MjREMHpzcWQybWVpTGZkSGZGOGNCQnV3bFowZ3dxeXl2bw?oc=5</t>
+          <t xml:space="preserve">https://era.gv.at/news-items/european-innovation-act-should-put-universities-at-the-heart-of-innovation-eua-says/</t>
         </is>
       </c>
     </row>
@@ -26826,27 +26826,27 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">R&amp;I needs to reduce dependencies on critical raw materials through advanced materials in electronics</t>
+          <t xml:space="preserve">EU's cybersecurity agency granted access to Mythos 5 AI model, Commission says</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-21</t>
+          <t xml:space="preserve">2026-09-10T08:56Z</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">JRC Publications Repository</t>
+          <t xml:space="preserve">Reuters</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main A</t>
+          <t xml:space="preserve">Main C</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
@@ -26861,7 +26861,7 @@
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Critical raw materials × R&amp;I / technology</t>
+          <t xml:space="preserve">EU-facing technology standards / regulatory alignment</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
@@ -26871,17 +26871,17 @@
       </c>
       <c r="K75" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: EU-facing technology standards / regulatory alignment</t>
         </is>
       </c>
       <c r="L75" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">JRC assesses 74 substitution, design, process, packaging and circularity options across five critical-material portfolios.</t>
+          <t xml:space="preserve">The EU cybersecurity agency received access to leading AI models to assess cybersecurity implications.</t>
         </is>
       </c>
       <c r="M75" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deployment bottlenecks identify where European R&amp;I capacity and infrastructure are needed.</t>
+          <t xml:space="preserve">Direct model access enables independent security testing and evidence for European AI and cyber-risk governance.</t>
         </is>
       </c>
       <c r="N75" s="3" t="inlineStr">
@@ -26906,12 +26906,12 @@
       </c>
       <c r="R75" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">COELHO, Fernando, OLIVEIRA, Filipa M., MOURDIKOUDIS, Stefanos, PENNINGTON, David</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="S75" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://publications.jrc.ec.europa.eu/repository/handle/JRC147525?mode=full</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMivAFBVV95cUxPRWVkQ1I1dzB2Wm10ZmloY0d5bW9PNEpSSnVTT0V5bHU0SXNsMnEyY1c0V2NmVnhzSm1qZ0JXZ1dsaHBDNkJmRXdzaWVaeks5ekhROVF0SjU3cGQ5VWRPc1NPRFd2UmtYRTJPZWVLamFvRjV0WmRnWk04UW13UUcwZnlGNFlORzd2cFUxZ056UkRJcEJaekZSMFM3MjREMHpzcWQybWVpTGZkSGZGOGNCQnV3bFowZ3dxeXl2bw?oc=5</t>
         </is>
       </c>
     </row>
@@ -26921,17 +26921,17 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Detecting and responding to cybersecurity incidents - Publications Office of the EU</t>
+          <t xml:space="preserve">R&amp;I needs to reduce dependencies on critical raw materials through advanced materials in electronics</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-22</t>
+          <t xml:space="preserve">2026-09-21</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU Publications Office</t>
+          <t xml:space="preserve">JRC Publications Repository</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
@@ -26956,7 +26956,7 @@
       </c>
       <c r="I76" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU-facing technology standards / regulatory alignment</t>
+          <t xml:space="preserve">Critical raw materials × R&amp;I / technology</t>
         </is>
       </c>
       <c r="J76" s="3" t="inlineStr">
@@ -26966,17 +26966,17 @@
       </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: EU-facing technology standards / regulatory alignment</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology</t>
         </is>
       </c>
       <c r="L76" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Detecting and responding to cybersecurity incidents - Publications Office of the EU. Cybersecurity is also a key element.</t>
+          <t xml:space="preserve">JRC assesses 74 substitution, design, process, packaging and circularity options across five critical-material portfolios.</t>
         </is>
       </c>
       <c r="M76" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Deployment bottlenecks identify where European R&amp;I capacity and infrastructure are needed.</t>
         </is>
       </c>
       <c r="N76" s="3" t="inlineStr">
@@ -27001,12 +27001,12 @@
       </c>
       <c r="R76" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU Publications Office</t>
+          <t xml:space="preserve">COELHO, Fernando, OLIVEIRA, Filipa M., MOURDIKOUDIS, Stefanos, PENNINGTON, David</t>
         </is>
       </c>
       <c r="S76" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://op.europa.eu/o/opportal-service/download-handler?identifier=692a9852-b703-11f1-81de-01aa75ed71a1&amp;format=pdf&amp;language=en&amp;productionSystem=cellar&amp;part=</t>
+          <t xml:space="preserve">https://publications.jrc.ec.europa.eu/repository/handle/JRC147525?mode=full</t>
         </is>
       </c>
     </row>
@@ -27016,27 +27016,27 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Allow dual-use research in next Horizon Europe, research ministers urge MEPs</t>
+          <t xml:space="preserve">Detecting and responding to cybersecurity incidents - Publications Office of the EU</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-28T21:34Z</t>
+          <t xml:space="preserve">2026-09-22</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Science|Business</t>
+          <t xml:space="preserve">EU Publications Office</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main C</t>
+          <t xml:space="preserve">Main A</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
@@ -27051,7 +27051,7 @@
       </c>
       <c r="I77" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research security / dual use</t>
+          <t xml:space="preserve">EU-facing technology standards / regulatory alignment</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr">
@@ -27061,17 +27061,17 @@
       </c>
       <c r="K77" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Research security / dual use</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: EU-facing technology standards / regulatory alignment</t>
         </is>
       </c>
       <c r="L77" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ministers from several European countries urged Parliament to support dual-use research in the next Horizon Europe.</t>
+          <t xml:space="preserve">Detecting and responding to cybersecurity incidents - Publications Office of the EU. Cybersecurity is also a key element.</t>
         </is>
       </c>
       <c r="M77" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Their joint intervention affects live negotiations over the scope of EU research funding.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="N77" s="3" t="inlineStr">
@@ -27096,12 +27096,12 @@
       </c>
       <c r="R77" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">EU Publications Office</t>
         </is>
       </c>
       <c r="S77" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMizAFBVV95cUxPMkhkTkprc0VSQUplbmhoOWx5UzJxQnYxQ0JqRXhaYlBrOWRqY2YwZnQ2cnlKTmpYcG9jZXB2MVVjSkIwTlYtRVc4ZTdoVkVDcGhKSmZCaVE0dk1NaWNvQjZDV19oTnNZbHpKMG5RMVRqV0ctR0dXSmFaR3oxaUZNcEotYU1fNGctUWZobl85aDVHd0dPUXpjZmRiUkpoWDBhZ1QwVzFMaWtJdkNFUmpFT3FZdFVic3lKWUdkVWhfRlNMVVFlQmxab1RmQ2w?oc=5</t>
+          <t xml:space="preserve">https://op.europa.eu/o/opportal-service/download-handler?identifier=692a9852-b703-11f1-81de-01aa75ed71a1&amp;format=pdf&amp;language=en&amp;productionSystem=cellar&amp;part=</t>
         </is>
       </c>
     </row>
@@ -27111,27 +27111,27 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reducing dependencies on Critical Raw Materials with advanced materials</t>
+          <t xml:space="preserve">Allow dual-use research in next Horizon Europe, research ministers urge MEPs</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-30</t>
+          <t xml:space="preserve">2026-09-28T21:34Z</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">JRC Publications Repository</t>
+          <t xml:space="preserve">Science|Business</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main A</t>
+          <t xml:space="preserve">Main C</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
@@ -27146,7 +27146,7 @@
       </c>
       <c r="I78" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Critical raw materials × R&amp;I / technology</t>
+          <t xml:space="preserve">Research security / dual use</t>
         </is>
       </c>
       <c r="J78" s="3" t="inlineStr">
@@ -27156,17 +27156,17 @@
       </c>
       <c r="K78" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Research security / dual use</t>
         </is>
       </c>
       <c r="L78" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">JRC identifies advanced-material substitution, efficiency and circularity as ways to reduce EU critical-material dependencies.</t>
+          <t xml:space="preserve">Ministers from several European countries urged Parliament to support dual-use research in the next Horizon Europe.</t>
         </is>
       </c>
       <c r="M78" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">It maps research and innovation needs tied directly to EU supply security and competitiveness.</t>
+          <t xml:space="preserve">Their joint intervention affects live negotiations over the scope of EU research funding.</t>
         </is>
       </c>
       <c r="N78" s="3" t="inlineStr">
@@ -27191,12 +27191,12 @@
       </c>
       <c r="R78" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">COELHO, Fernando, PENNINGTON, David, SALA, Serenella</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="S78" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://publications.jrc.ec.europa.eu/repository/handle/JRC148453</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMizAFBVV95cUxPMkhkTkprc0VSQUplbmhoOWx5UzJxQnYxQ0JqRXhaYlBrOWRqY2YwZnQ2cnlKTmpYcG9jZXB2MVVjSkIwTlYtRVc4ZTdoVkVDcGhKSmZCaVE0dk1NaWNvQjZDV19oTnNZbHpKMG5RMVRqV0ctR0dXSmFaR3oxaUZNcEotYU1fNGctUWZobl85aDVHd0dPUXpjZmRiUkpoWDBhZ1QwVzFMaWtJdkNFUmpFT3FZdFVic3lKWUdkVWhfRlNMVVFlQmxab1RmQ2w?oc=5</t>
         </is>
       </c>
     </row>
@@ -27206,27 +27206,27 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Europe’s carmakers compete with AI for chips and critical materials</t>
+          <t xml:space="preserve">Reducing dependencies on Critical Raw Materials with advanced materials</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-30T10:39Z</t>
+          <t xml:space="preserve">2026-09-30</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Euronews</t>
+          <t xml:space="preserve">JRC Publications Repository</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main C</t>
+          <t xml:space="preserve">Main A</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
       <c r="G79" s="3" t="inlineStr">
@@ -27256,12 +27256,12 @@
       </c>
       <c r="L79" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A new report says European carmakers increasingly compete with AI and data centres for chips and critical materials.</t>
+          <t xml:space="preserve">JRC identifies advanced-material substitution, efficiency and circularity as ways to reduce EU critical-material dependencies.</t>
         </is>
       </c>
       <c r="M79" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The finding links European industrial technology capacity to constrained strategic inputs.</t>
+          <t xml:space="preserve">It maps research and innovation needs tied directly to EU supply security and competitiveness.</t>
         </is>
       </c>
       <c r="N79" s="3" t="inlineStr">
@@ -27286,12 +27286,12 @@
       </c>
       <c r="R79" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">COELHO, Fernando, PENNINGTON, David, SALA, Serenella</t>
         </is>
       </c>
       <c r="S79" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMiqAFBVV95cUxQU1BaSVprUWJOWWxrZGM1R00xemZnOFlEMUVxSG15UUV4a3VzUWZOaFpiYk8xaFJKSUxpTXpXMy1lcmswbGdzYU1zVGxfMEt0eS1vUWV0TDdYeDNJNWhucXdxQlVPbzdMamJmOFBNcVZzanJoNVhRVVU1T2JHbWI1MXNaYy1RT3VSNy1yNDVtWGxyQkcwTkpLWVFDNzQwcUZYUXMxRnZfMjI?oc=5</t>
+          <t xml:space="preserve">https://publications.jrc.ec.europa.eu/repository/handle/JRC148453</t>
         </is>
       </c>
     </row>
@@ -27301,27 +27301,27 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">R&amp;I needs to reduce critical raw materials through advanced materials in construction</t>
+          <t xml:space="preserve">Europe’s carmakers compete with AI for chips and critical materials</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-09-30T10:39Z</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">JRC Publications Repository</t>
+          <t xml:space="preserve">Euronews</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main A</t>
+          <t xml:space="preserve">Main C</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
@@ -27351,12 +27351,12 @@
       </c>
       <c r="L80" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">JRC compares 43 substitution, design, process and circularity routes for critical materials used in construction.</t>
+          <t xml:space="preserve">A new report says European carmakers increasingly compete with AI and data centres for chips and critical materials.</t>
         </is>
       </c>
       <c r="M80" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The report identifies qualification, pilot-line and scale-up constraints for EU deployment.</t>
+          <t xml:space="preserve">The finding links European industrial technology capacity to constrained strategic inputs.</t>
         </is>
       </c>
       <c r="N80" s="3" t="inlineStr">
@@ -27381,12 +27381,12 @@
       </c>
       <c r="R80" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">HAVERIKU, Sara, LAMPERTI, TORNAGHI Marco</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="S80" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://publications.jrc.ec.europa.eu/repository/handle/JRC147428?mode=full</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMiqAFBVV95cUxQU1BaSVprUWJOWWxrZGM1R00xemZnOFlEMUVxSG15UUV4a3VzUWZOaFpiYk8xaFJKSUxpTXpXMy1lcmswbGdzYU1zVGxfMEt0eS1vUWV0TDdYeDNJNWhucXdxQlVPbzdMamJmOFBNcVZzanJoNVhRVVU1T2JHbWI1MXNaYy1RT3VSNy1yNDVtWGxyQkcwTkpLWVFDNzQwcUZYUXMxRnZfMjI?oc=5</t>
         </is>
       </c>
     </row>
@@ -27396,27 +27396,27 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dual-use restrictions risk holding back research, Nordic universities say</t>
+          <t xml:space="preserve">R&amp;I needs to reduce critical raw materials through advanced materials in construction</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01T14:50Z</t>
+          <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Science|Business</t>
+          <t xml:space="preserve">JRC Publications Repository</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main C</t>
+          <t xml:space="preserve">Main A</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -27431,27 +27431,27 @@
       </c>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research security / dual use</t>
+          <t xml:space="preserve">Critical raw materials × R&amp;I / technology</t>
         </is>
       </c>
       <c r="J81" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Universities / research institutions</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K81" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Research security / dual use</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology</t>
         </is>
       </c>
       <c r="L81" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nordic university leaders warned that overly restrictive dual-use rules could exclude scientifically valuable Horizon Europe research.</t>
+          <t xml:space="preserve">JRC compares 43 substitution, design, process and circularity routes for critical materials used in construction.</t>
         </is>
       </c>
       <c r="M81" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Their intervention feeds an active EU decision over the scope of the next research programme.</t>
+          <t xml:space="preserve">The report identifies qualification, pilot-line and scale-up constraints for EU deployment.</t>
         </is>
       </c>
       <c r="N81" s="3" t="inlineStr">
@@ -27476,12 +27476,12 @@
       </c>
       <c r="R81" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">HAVERIKU, Sara, LAMPERTI, TORNAGHI Marco</t>
         </is>
       </c>
       <c r="S81" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMivAFBVV95cUxPNl9UZUx6VWZ4bmlmeUg2a2xjUV9DdTBBaFJEM2o4emtxaHNHMnFvcnNicHdXZkxET0ZYMWkyckNXNVZtamZsREhuQUVYLVFrQ0dTT1pRb1M5N2F5LVhlVGU2cWlpcndxbDhjSV9tZThzRGlpWTBHY3FYdHU3NE1wOGpGNng3aUpBWVFXQU1sNVBlU05CeWJ2UGNjWGVIMng1dEtJWWY5M0ZtZnNHajNxcFZKdHRpRGYwb2F4Sg?oc=5</t>
+          <t xml:space="preserve">https://publications.jrc.ec.europa.eu/repository/handle/JRC147428?mode=full</t>
         </is>
       </c>
     </row>
@@ -27491,17 +27491,17 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Horizon Europe launches a new research and innovation call on nature</t>
+          <t xml:space="preserve">Dual-use restrictions risk holding back research, Nordic universities say</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-02T08:13Z</t>
+          <t xml:space="preserve">2026-10-01T14:50Z</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU Research &amp; Innovation</t>
+          <t xml:space="preserve">Science|Business</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
@@ -27526,27 +27526,27 @@
       </c>
       <c r="I82" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Research security / dual use</t>
         </is>
       </c>
       <c r="J82" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Universities / research institutions</t>
         </is>
       </c>
       <c r="K82" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: EU external R&amp;I partnerships / enlargement</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Research security / dual use</t>
         </is>
       </c>
       <c r="L82" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Commission announced a €230 million Horizon Europe nature call covering ten biodiversity research topics.</t>
+          <t xml:space="preserve">Nordic university leaders warned that overly restrictive dual-use rules could exclude scientifically valuable Horizon Europe research.</t>
         </is>
       </c>
       <c r="M82" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The new call explicitly increases R&amp;I funding for European biodiversity, monitoring and ecosystem restoration.</t>
+          <t xml:space="preserve">Their intervention feeds an active EU decision over the scope of the next research programme.</t>
         </is>
       </c>
       <c r="N82" s="3" t="inlineStr">
@@ -27576,7 +27576,7 @@
       </c>
       <c r="S82" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMi8gFBVV95cUxNVzJrbnB6clF0YzUzZmkxUUZ3V2hpV0xfN2lILXFyOGFoRExET1lvUzdKakhKR1NyS2pQdWVnSVhkWV9kM3U2NGtjaEhTeURmaXJNYmJqTDNzVUFiM0VDYnFhNW1pMmZlb3pHMkVqemkyNllRTW5OSDdPQjZwME1xODNzeHRjdDFuTF9qT0MtMWZwSWwxRC1UX25wRWxfLWUydDhITnVJcTYwQ1ptZ1JoX2lYdC0ta3l5NVBuYVN2Q1lwQndzUnZiSnJEbDhQenZVT3M4WUdvaWdmMlVQYlpwQ3N5X3NPTXNfRlhsc19DX0I5Zw?oc=5</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMivAFBVV95cUxPNl9UZUx6VWZ4bmlmeUg2a2xjUV9DdTBBaFJEM2o4emtxaHNHMnFvcnNicHdXZkxET0ZYMWkyckNXNVZtamZsREhuQUVYLVFrQ0dTT1pRb1M5N2F5LVhlVGU2cWlpcndxbDhjSV9tZThzRGlpWTBHY3FYdHU3NE1wOGpGNng3aUpBWVFXQU1sNVBlU05CeWJ2UGNjWGVIMng1dEtJWWY5M0ZtZnNHajNxcFZKdHRpRGYwb2F4Sg?oc=5</t>
         </is>
       </c>
     </row>
@@ -27586,17 +27586,17 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU weighs mirroring Donald Trump in securing critical minerals</t>
+          <t xml:space="preserve">Horizon Europe launches a new research and innovation call on nature</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-26T05:00Z</t>
+          <t xml:space="preserve">2026-10-02T08:13Z</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Financial Times</t>
+          <t xml:space="preserve">EU Research &amp; Innovation</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
@@ -27621,7 +27621,7 @@
       </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Critical raw materials × R&amp;I / technology</t>
+          <t xml:space="preserve">EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="J83" s="3" t="inlineStr">
@@ -27631,17 +27631,17 @@
       </c>
       <c r="K83" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: EU external R&amp;I partnerships / enlargement</t>
         </is>
       </c>
       <c r="L83" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">European lawmakers backed a proposed Critical Raw Materials Centre able to acquire stakes in mineral projects and coordinate stockpiles.</t>
+          <t xml:space="preserve">The Commission announced a €230 million Horizon Europe nature call covering ten biodiversity research topics.</t>
         </is>
       </c>
       <c r="M83" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposed investment and stockpiling instruments would address strategic material inputs for European clean technology, batteries and defence innovation.</t>
+          <t xml:space="preserve">The new call explicitly increases R&amp;I funding for European biodiversity, monitoring and ecosystem restoration.</t>
         </is>
       </c>
       <c r="N83" s="3" t="inlineStr">
@@ -27671,27 +27671,27 @@
       </c>
       <c r="S83" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMihAFBVV95cUxPTkh2ek1Gc3lfdzhmdi1xc25PbEt1UHVLMjdXeHN1V1BuLTR3RHhLVDhhWFAxZXdCM3ZrYXA1c05CX1hrTkZabEt2eGUxSGRfQXRZWGdCTFNIZl9iMnVNT3c4UTFoMTZyZmRoTlMxZHJRSzFRSlo4dzV4UkhPRHNtekZGS3I?oc=5</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMi8gFBVV95cUxNVzJrbnB6clF0YzUzZmkxUUZ3V2hpV0xfN2lILXFyOGFoRExET1lvUzdKakhKR1NyS2pQdWVnSVhkWV9kM3U2NGtjaEhTeURmaXJNYmJqTDNzVUFiM0VDYnFhNW1pMmZlb3pHMkVqemkyNllRTW5OSDdPQjZwME1xODNzeHRjdDFuTF9qT0MtMWZwSWwxRC1UX25wRWxfLWUydDhITnVJcTYwQ1ptZ1JoX2lYdC0ta3l5NVBuYVN2Q1lwQndzUnZiSnJEbDhQenZVT3M4WUdvaWdmMlVQYlpwQ3N5X3NPTXNfRlhsc19DX0I5Zw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="3">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU-China trade and investment relations</t>
+          <t xml:space="preserve">EU weighs mirroring Donald Trump in securing critical minerals</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-28T16:04Z</t>
+          <t xml:space="preserve">2026-10-26T05:00Z</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">European Parliament</t>
+          <t xml:space="preserve">Financial Times</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
@@ -27706,17 +27706,17 @@
       </c>
       <c r="G84" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">China</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asia &amp; Pacific</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I84" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transnational R&amp;I and innovation policy</t>
+          <t xml:space="preserve">Critical raw materials × R&amp;I / technology</t>
         </is>
       </c>
       <c r="J84" s="3" t="inlineStr">
@@ -27726,17 +27726,17 @@
       </c>
       <c r="K84" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Region: China; issue: Transnational R&amp;I and innovation policy</t>
+          <t xml:space="preserve">Region: cross-regional / ABNJ; issue: Critical raw materials × R&amp;I / technology</t>
         </is>
       </c>
       <c r="L84" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EU-China trade and investment relations. The repository record provides substantive source material sufficient for a terminal Deep Scan.</t>
+          <t xml:space="preserve">European lawmakers backed a proposed Critical Raw Materials Centre able to acquire stakes in mineral projects and coordinate stockpiles.</t>
         </is>
       </c>
       <c r="M84" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Proposed investment and stockpiling instruments would address strategic material inputs for European clean technology, batteries and defence innovation.</t>
         </is>
       </c>
       <c r="N84" s="3" t="inlineStr">
@@ -27766,7 +27766,7 @@
       </c>
       <c r="S84" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://news.google.com/rss/articles/CBMifkFVX3lxTE5na2d5djZmZnloSXVwUGVEeTRhOE9rLVFUSUE0VXBlaGUyZUFNdk5wSm9JMEZ1VDd6Yk5CakJDdV9wdjhQYi1FNFd5VkhITWpPMlo0YkdJUkd4Ti1ueUJXdVhDam1yUEZTMnhIcmRQWm4tTE80MzlRNUhiUGlSdw?oc=5</t>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMihAFBVV95cUxPTkh2ek1Gc3lfdzhmdi1xc25PbEt1UHVLMjdXeHN1V1BuLTR3RHhLVDhhWFAxZXdCM3ZrYXA1c05CX1hrTkZabEt2eGUxSGRfQXRZWGdCTFNIZl9iMnVNT3c4UTFoMTZyZmRoTlMxZHJRSzFRSlo4dzV4UkhPRHNtekZGS3I?oc=5</t>
         </is>
       </c>
     </row>
@@ -27776,97 +27776,192 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">EU-China trade and investment relations</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28T16:04Z</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">European Parliament</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Main C</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">China</t>
+        </is>
+      </c>
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asia &amp; Pacific</t>
+        </is>
+      </c>
+      <c r="I85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transnational R&amp;I and innovation policy</t>
+        </is>
+      </c>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Region: China; issue: Transnational R&amp;I and innovation policy</t>
+        </is>
+      </c>
+      <c r="L85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EU-China trade and investment relations. The repository record provides substantive source material sufficient for a terminal Deep Scan.</t>
+        </is>
+      </c>
+      <c r="M85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">keep</t>
+        </is>
+      </c>
+      <c r="O85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Review / awaiting authoritative retention</t>
+        </is>
+      </c>
+      <c r="P85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Q85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://news.google.com/rss/articles/CBMifkFVX3lxTE5na2d5djZmZnloSXVwUGVEeTRhOE9rLVFUSUE0VXBlaGUyZUFNdk5wSm9JMEZ1VDd6Yk5CakJDdV9wdjhQYi1FNFd5VkhITWpPMlo0YkdJUkd4Ti1ueUJXdVhDam1yUEZTMnhIcmRQWm4tTE80MzlRNUhiUGlSdw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3">
+        <v>58</v>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">EU-China political relations | 05-10-2026 | News</t>
         </is>
       </c>
-      <c r="C85" s="3" t="inlineStr">
+      <c r="C86" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01T13:52Z</t>
         </is>
       </c>
-      <c r="D85" s="3" t="inlineStr">
+      <c r="D86" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">European Parliament</t>
         </is>
       </c>
-      <c r="E85" s="3" t="inlineStr">
+      <c r="E86" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Main C</t>
         </is>
       </c>
-      <c r="F85" s="3" t="inlineStr">
+      <c r="F86" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">C</t>
         </is>
       </c>
-      <c r="G85" s="3" t="inlineStr">
+      <c r="G86" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">China</t>
         </is>
       </c>
-      <c r="H85" s="3" t="inlineStr">
+      <c r="H86" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Asia &amp; Pacific</t>
         </is>
       </c>
-      <c r="I85" s="3" t="inlineStr">
+      <c r="I86" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Transnational R&amp;I and innovation policy</t>
         </is>
       </c>
-      <c r="J85" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K85" s="3" t="inlineStr">
+      <c r="J86" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K86" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Region: China; issue: Transnational R&amp;I and innovation policy</t>
         </is>
       </c>
-      <c r="L85" s="3" t="inlineStr">
+      <c r="L86" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">EU-China political relations | 05-10-2026 | News.</t>
         </is>
       </c>
-      <c r="M85" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N85" s="3" t="inlineStr">
+      <c r="M86" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N86" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">keep</t>
         </is>
       </c>
-      <c r="O85" s="3" t="inlineStr">
+      <c r="O86" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Review / awaiting authoritative retention</t>
         </is>
       </c>
-      <c r="P85" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="Q85" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="R85" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="S85" s="3" t="inlineStr">
+      <c r="P86" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Q86" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R86" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S86" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">https://news.google.com/rss/articles/CBMiogFBVV95cUxQWmlaa2hLZEw1UjBQMG9tTzMxWC1BMzBJRnkwTmhuajBMSHNrSUdYTWh4bXd5N0lVWlhhMTNHLUNRaS1id1JYZU1PUVljMnU5X2ZBc0VtN2g1TUtFeUU4dEhzTGYtdG5OeGFFeTZIb3lhVGREN3BjWElOZ0s0SnBVOFJqVkl5anVYV0tYdzVjS1pYSm9BX3hUUVN4WWdRX05WMXc?oc=5</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S85"/>
+  <autoFilter ref="A1:S86"/>
 </worksheet>
 </file>
 
@@ -28888,7 +28983,7 @@
         <v>138</v>
       </c>
       <c r="D56" s="3">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="57">
@@ -28924,7 +29019,7 @@
         <v>2</v>
       </c>
       <c r="D58" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
@@ -29061,7 +29156,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-31T02:22:57+00:00</t>
+          <t xml:space="preserve">2026-10-31T06:24:03+00:00</t>
         </is>
       </c>
     </row>
@@ -29082,7 +29177,7 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6">

</xml_diff>